<commit_message>
build: v2 Welcome Book Start tab — hero + 3-card + Quick Start + Get Started + progress dashboard
</commit_message>
<xml_diff>
--- a/templates/_masters/GST-001-welcome-book-BLANK.xlsx
+++ b/templates/_masters/GST-001-welcome-book-BLANK.xlsx
@@ -20,7 +20,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bonus" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="× Host Notes" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Start'!$A$1:$L$52</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -28,7 +30,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,16 +38,105 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Georgia"/>
+      <color rgb="00F6EFE2"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="00F6EFE2"/>
+      <sz val="36"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <i val="1"/>
+      <color rgb="00C9A24B"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="00C9A24B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="0012304E"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="0012304E"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="002B2B2B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="00F6EFE2"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="0012304E"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="00C9A24B"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C9A24B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="006B7280"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00C9A24B"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0012304E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F6EFE2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFE5D0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -53,12 +144,92 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <top style="medium">
+        <color rgb="00C9A24B"/>
+      </top>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00C9A24B"/>
+      </left>
+      <right style="medium">
+        <color rgb="00C9A24B"/>
+      </right>
+      <top style="medium">
+        <color rgb="00C9A24B"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00C9A24B"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="00C9A24B"/>
+      </top>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,12 +594,576 @@
   <sheetPr>
     <tabColor rgb="0012304E"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>The STR Ledger</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Welcome Book</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Welcome books that earn 5-stars.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="1" t="n"/>
+      <c r="C6" s="1" t="n"/>
+      <c r="D6" s="1" t="n"/>
+      <c r="E6" s="1" t="n"/>
+      <c r="F6" s="1" t="n"/>
+      <c r="G6" s="1" t="n"/>
+      <c r="H6" s="1" t="n"/>
+      <c r="I6" s="1" t="n"/>
+      <c r="J6" s="1" t="n"/>
+      <c r="K6" s="1" t="n"/>
+      <c r="L6" s="1" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>GST-001 · v2.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="1" t="n"/>
+      <c r="B8" s="1" t="n"/>
+      <c r="C8" s="1" t="n"/>
+      <c r="D8" s="1" t="n"/>
+      <c r="E8" s="1" t="n"/>
+      <c r="F8" s="1" t="n"/>
+      <c r="G8" s="1" t="n"/>
+      <c r="H8" s="1" t="n"/>
+      <c r="I8" s="1" t="n"/>
+      <c r="J8" s="1" t="n"/>
+      <c r="K8" s="1" t="n"/>
+      <c r="L8" s="1" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="n"/>
+      <c r="K10" s="6" t="n"/>
+      <c r="L10" s="6" t="n"/>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>What you'll build in the next 15 minutes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="n"/>
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>📖 PRINT</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>📱 QR CODE</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>✉ EMAIL PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Spiral-bound binder for the kitchen counter.</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Scan on arrival — view on the guest's phone.</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>Send ahead of check-in. One page, every tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1"/>
+    <row r="16" ht="22" customHeight="1"/>
+    <row r="17" ht="22" customHeight="1"/>
+    <row r="18" ht="22" customHeight="1"/>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="6" t="n"/>
+      <c r="J19" s="6" t="n"/>
+      <c r="K19" s="6" t="n"/>
+      <c r="L19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="6" t="n"/>
+      <c r="J20" s="6" t="n"/>
+      <c r="K20" s="6" t="n"/>
+      <c r="L20" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="n"/>
+      <c r="B22" s="10" t="n"/>
+      <c r="C22" s="10" t="n"/>
+      <c r="D22" s="10" t="n"/>
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="10" t="n"/>
+      <c r="G22" s="10" t="n"/>
+      <c r="H22" s="10" t="n"/>
+      <c r="I22" s="10" t="n"/>
+      <c r="J22" s="10" t="n"/>
+      <c r="K22" s="10" t="n"/>
+      <c r="L22" s="10" t="n"/>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>Quick Start — be done in 5 minutes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="n"/>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>① Property name + host phone</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="n"/>
+      <c r="H24" s="12" t="inlineStr">
+        <is>
+          <t>④ Checkout time</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="n"/>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>② WiFi network + password</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="n"/>
+      <c r="H25" s="12" t="inlineStr">
+        <is>
+          <t>⑤ Hospital + 911 note</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="n"/>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>③ Trash pickup day</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="n"/>
+      <c r="H26" s="10" t="n"/>
+      <c r="I26" s="10" t="n"/>
+      <c r="J26" s="10" t="n"/>
+      <c r="K26" s="10" t="n"/>
+      <c r="L26" s="10" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="n"/>
+      <c r="B27" s="10" t="n"/>
+      <c r="C27" s="10" t="n"/>
+      <c r="D27" s="10" t="n"/>
+      <c r="E27" s="10" t="n"/>
+      <c r="F27" s="10" t="n"/>
+      <c r="G27" s="10" t="n"/>
+      <c r="H27" s="10" t="n"/>
+      <c r="I27" s="10" t="n"/>
+      <c r="J27" s="10" t="n"/>
+      <c r="K27" s="10" t="n"/>
+      <c r="L27" s="10" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="n"/>
+      <c r="B28" s="10" t="n"/>
+      <c r="C28" s="10" t="n"/>
+      <c r="D28" s="10" t="n"/>
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="10" t="n"/>
+      <c r="G28" s="10" t="n"/>
+      <c r="H28" s="10" t="n"/>
+      <c r="I28" s="10" t="n"/>
+      <c r="J28" s="10" t="n"/>
+      <c r="K28" s="10" t="n"/>
+      <c r="L28" s="10" t="n"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="13">
+        <f>HYPERLINK("#'Property'!A5", "GET STARTED — FILL YOUR PROPERTY INFO  →")</f>
+        <v/>
+      </c>
+      <c r="B30" s="14" t="n"/>
+      <c r="C30" s="14" t="n"/>
+      <c r="D30" s="14" t="n"/>
+      <c r="E30" s="14" t="n"/>
+      <c r="F30" s="14" t="n"/>
+      <c r="G30" s="14" t="n"/>
+      <c r="H30" s="14" t="n"/>
+      <c r="I30" s="14" t="n"/>
+      <c r="J30" s="14" t="n"/>
+      <c r="K30" s="14" t="n"/>
+      <c r="L30" s="14" t="n"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="14" t="n"/>
+      <c r="B31" s="14" t="n"/>
+      <c r="C31" s="14" t="n"/>
+      <c r="D31" s="14" t="n"/>
+      <c r="E31" s="14" t="n"/>
+      <c r="F31" s="14" t="n"/>
+      <c r="G31" s="14" t="n"/>
+      <c r="H31" s="14" t="n"/>
+      <c r="I31" s="14" t="n"/>
+      <c r="J31" s="14" t="n"/>
+      <c r="K31" s="14" t="n"/>
+      <c r="L31" s="14" t="n"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="14" t="n"/>
+      <c r="B32" s="14" t="n"/>
+      <c r="C32" s="14" t="n"/>
+      <c r="D32" s="14" t="n"/>
+      <c r="E32" s="14" t="n"/>
+      <c r="F32" s="14" t="n"/>
+      <c r="G32" s="14" t="n"/>
+      <c r="H32" s="14" t="n"/>
+      <c r="I32" s="14" t="n"/>
+      <c r="J32" s="14" t="n"/>
+      <c r="K32" s="14" t="n"/>
+      <c r="L32" s="14" t="n"/>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="14" t="n"/>
+      <c r="B33" s="14" t="n"/>
+      <c r="C33" s="14" t="n"/>
+      <c r="D33" s="14" t="n"/>
+      <c r="E33" s="14" t="n"/>
+      <c r="F33" s="14" t="n"/>
+      <c r="G33" s="14" t="n"/>
+      <c r="H33" s="14" t="n"/>
+      <c r="I33" s="14" t="n"/>
+      <c r="J33" s="14" t="n"/>
+      <c r="K33" s="14" t="n"/>
+      <c r="L33" s="14" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="15" t="inlineStr">
+        <is>
+          <t>Progress:</t>
+        </is>
+      </c>
+      <c r="G36" s="16">
+        <f>TEXT((COUNTA('Property'!B5:B12) + COUNTA('Arrival'!B5:B11) + COUNTA('WiFi + Tech'!B5:B12) + COUNTA('House Rules'!B5:B11) + COUNTA('Local Guide'!B6:E25) + COUNTA('Trash'!B5:B11) + COUNTA('Departure'!B5:B10) + COUNTA('Emergency'!B5:B13))/132, "0%") &amp; " complete"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>① Property Info</t>
+        </is>
+      </c>
+      <c r="G38" s="18">
+        <f>IF(COUNTA('Property'!B5:B12)=8,"✅ Done",IF(COUNTA('Property'!B5:B12)=0,"⏳ Empty","⏳ "&amp;COUNTA('Property'!B5:B12)&amp;" of 8"))</f>
+        <v/>
+      </c>
+      <c r="K38" s="19">
+        <f>HYPERLINK("#'Property'!A5","→ go")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>② Arrival</t>
+        </is>
+      </c>
+      <c r="G39" s="18">
+        <f>IF(COUNTA('Arrival'!B5:B11)=7,"✅ Done",IF(COUNTA('Arrival'!B5:B11)=0,"⏳ Empty","⏳ "&amp;COUNTA('Arrival'!B5:B11)&amp;" of 7"))</f>
+        <v/>
+      </c>
+      <c r="K39" s="19">
+        <f>HYPERLINK("#'Arrival'!A5","→ go")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>③ WiFi + Tech</t>
+        </is>
+      </c>
+      <c r="G40" s="18">
+        <f>IF(COUNTA('WiFi + Tech'!B5:B12)=8,"✅ Done",IF(COUNTA('WiFi + Tech'!B5:B12)=0,"⏳ Empty","⏳ "&amp;COUNTA('WiFi + Tech'!B5:B12)&amp;" of 8"))</f>
+        <v/>
+      </c>
+      <c r="K40" s="19">
+        <f>HYPERLINK("#'WiFi + Tech'!A5","→ go")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="17" t="inlineStr">
+        <is>
+          <t>④ House Rules</t>
+        </is>
+      </c>
+      <c r="G41" s="18">
+        <f>IF(COUNTA('House Rules'!B5:B11)=7,"✅ Done",IF(COUNTA('House Rules'!B5:B11)=0,"⏳ Empty","⏳ "&amp;COUNTA('House Rules'!B5:B11)&amp;" of 7"))</f>
+        <v/>
+      </c>
+      <c r="K41" s="19">
+        <f>HYPERLINK("#'House Rules'!A5","→ go")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="17" t="inlineStr">
+        <is>
+          <t>⑤ Local Guide</t>
+        </is>
+      </c>
+      <c r="G42" s="18">
+        <f>IF(COUNTA('Local Guide'!B6:E25)=80,"✅ Done",IF(COUNTA('Local Guide'!B6:E25)=0,"⏳ Empty","⏳ "&amp;COUNTA('Local Guide'!B6:E25)&amp;" of 80"))</f>
+        <v/>
+      </c>
+      <c r="K42" s="19">
+        <f>HYPERLINK("#'Local Guide'!A5","→ go")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>⑥ Trash</t>
+        </is>
+      </c>
+      <c r="G43" s="18">
+        <f>IF(COUNTA('Trash'!B5:B11)=7,"✅ Done",IF(COUNTA('Trash'!B5:B11)=0,"⏳ Empty","⏳ "&amp;COUNTA('Trash'!B5:B11)&amp;" of 7"))</f>
+        <v/>
+      </c>
+      <c r="K43" s="19">
+        <f>HYPERLINK("#'Trash'!A5","→ go")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="17" t="inlineStr">
+        <is>
+          <t>⑦ Departure</t>
+        </is>
+      </c>
+      <c r="G44" s="18">
+        <f>IF(COUNTA('Departure'!B5:B10)=6,"✅ Done",IF(COUNTA('Departure'!B5:B10)=0,"⏳ Empty","⏳ "&amp;COUNTA('Departure'!B5:B10)&amp;" of 6"))</f>
+        <v/>
+      </c>
+      <c r="K44" s="19">
+        <f>HYPERLINK("#'Departure'!A5","→ go")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="17" t="inlineStr">
+        <is>
+          <t>⑧ Emergency</t>
+        </is>
+      </c>
+      <c r="G45" s="18">
+        <f>IF(COUNTA('Emergency'!B5:B13)=9,"✅ Done",IF(COUNTA('Emergency'!B5:B13)=0,"⏳ Empty","⏳ "&amp;COUNTA('Emergency'!B5:B13)&amp;" of 9"))</f>
+        <v/>
+      </c>
+      <c r="K45" s="19">
+        <f>HYPERLINK("#'Emergency'!A5","→ go")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="20" t="n"/>
+      <c r="B49" s="20" t="n"/>
+      <c r="C49" s="20" t="n"/>
+      <c r="D49" s="20" t="n"/>
+      <c r="E49" s="20" t="n"/>
+      <c r="F49" s="20" t="n"/>
+      <c r="G49" s="20" t="n"/>
+      <c r="H49" s="20" t="n"/>
+      <c r="I49" s="20" t="n"/>
+      <c r="J49" s="20" t="n"/>
+      <c r="K49" s="20" t="n"/>
+      <c r="L49" s="20" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="21" t="inlineStr">
+        <is>
+          <t>Questions? hello@thestrledger.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="22" t="inlineStr">
+        <is>
+          <t>Free updates forever · v2.0 · Released 2026-05</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="46">
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="K45:L45"/>
+    <mergeCell ref="A14:D18"/>
+    <mergeCell ref="G41:J41"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="I14:L18"/>
+    <mergeCell ref="A50:L50"/>
+    <mergeCell ref="G44:J44"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="I13:L13"/>
+    <mergeCell ref="G40:J40"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="H25:L25"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A23:L23"/>
+    <mergeCell ref="G43:J43"/>
+    <mergeCell ref="K44:L44"/>
+    <mergeCell ref="K41:L41"/>
+    <mergeCell ref="K40:L40"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="G42:J42"/>
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A43:F43"/>
+    <mergeCell ref="K43:L43"/>
+    <mergeCell ref="G39:J39"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="A30:L33"/>
+    <mergeCell ref="K42:L42"/>
+    <mergeCell ref="G38:J38"/>
+    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="K39:L39"/>
+    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="E14:H18"/>
+    <mergeCell ref="E13:H13"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="G36:L36"/>
+    <mergeCell ref="A11:L11"/>
+    <mergeCell ref="K38:L38"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="A51:L51"/>
+    <mergeCell ref="H24:L24"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="G45:J45"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
build: v2 Welcome Book — 8 input tabs with card-grouped layout, dropdowns, cross-sheet formulas
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/_masters/GST-001-welcome-book-BLANK.xlsx
+++ b/templates/_masters/GST-001-welcome-book-BLANK.xlsx
@@ -22,6 +22,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Start'!$A$1:$L$52</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'Local Guide'!$A$1:$E$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="8">'Emergency'!$A$1:$L$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -30,7 +32,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -112,8 +114,74 @@
       <color rgb="00C9A24B"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="00C9A24B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="0012304E"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="00F6EFE2"/>
+      <sz val="28"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <i val="1"/>
+      <color rgb="00C9A24B"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="002B2B2B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="0012304E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002B2B2B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0012304E"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="002B2B2B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="00B91C1C"/>
+      <sz val="22"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -135,8 +203,33 @@
         <fgColor rgb="00EFE5D0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C9A24B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2C884"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF7D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE8E8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -168,11 +261,179 @@
         <color rgb="00C9A24B"/>
       </top>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="0012304E"/>
+      </left>
+      <right style="medium">
+        <color rgb="0012304E"/>
+      </right>
+      <top style="medium">
+        <color rgb="0012304E"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="0012304E"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9A24B"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9A24B"/>
+      </top>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9A24B"/>
+      </top>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9A24B"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9A24B"/>
+      </top>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9A24B"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C9A24B"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C9A24B"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9A24B"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C9A24B"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9A24B"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9A24B"/>
+      </right>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9A24B"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C9A24B"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9A24B"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9A24B"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9A24B"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9A24B"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9A24B"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9A24B"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9A24B"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9A24B"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9A24B"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9A24B"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="0012304E"/>
+      </left>
+      <right style="thin">
+        <color rgb="0012304E"/>
+      </right>
+      <top style="thin">
+        <color rgb="0012304E"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="0012304E"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9A24B"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00B91C1C"/>
+      </left>
+      <right style="medium">
+        <color rgb="00B91C1C"/>
+      </right>
+      <top style="medium">
+        <color rgb="00B91C1C"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00B91C1C"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -229,6 +490,94 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1216,9 +1565,414 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="8" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="13">
+        <f>HYPERLINK("#'Start'!A1", "← START")</f>
+        <v/>
+      </c>
+      <c r="B2" s="14" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="23" t="inlineStr">
+        <is>
+          <t>SECTION 1 OF 8</t>
+        </is>
+      </c>
+      <c r="J2" s="24">
+        <f>HYPERLINK("#'Arrival'!A5", "NEXT →")</f>
+        <v/>
+      </c>
+      <c r="K2" s="25" t="n"/>
+      <c r="L2" s="25" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>Property Info</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>Who you are and where they're staying.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="6" customHeight="1">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Fill the highlighted fields below. The 'Review &amp; Print' tab (last) shows what your guest will see.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>IDENTITY</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Property name:</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="n"/>
+      <c r="C10" s="31" t="n"/>
+      <c r="D10" s="32" t="n"/>
+      <c r="E10" s="31" t="n"/>
+      <c r="F10" s="31" t="n"/>
+      <c r="G10" s="31" t="n"/>
+      <c r="H10" s="31" t="n"/>
+      <c r="I10" s="31" t="n"/>
+      <c r="J10" s="31" t="n"/>
+      <c r="K10" s="31" t="n"/>
+      <c r="L10" s="33" t="n"/>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="34" t="inlineStr">
+        <is>
+          <t>Host first name:</t>
+        </is>
+      </c>
+      <c r="B11" s="35" t="n"/>
+      <c r="C11" s="35" t="n"/>
+      <c r="D11" s="36" t="n"/>
+      <c r="E11" s="35" t="n"/>
+      <c r="F11" s="35" t="n"/>
+      <c r="G11" s="35" t="n"/>
+      <c r="H11" s="35" t="n"/>
+      <c r="I11" s="35" t="n"/>
+      <c r="J11" s="35" t="n"/>
+      <c r="K11" s="35" t="n"/>
+      <c r="L11" s="37" t="n"/>
+    </row>
+    <row r="12" ht="12" customHeight="1">
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="n"/>
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>GUEST DETAILS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>Host phone (text preferred):</t>
+        </is>
+      </c>
+      <c r="B14" s="31" t="n"/>
+      <c r="C14" s="31" t="n"/>
+      <c r="D14" s="32" t="n"/>
+      <c r="E14" s="31" t="n"/>
+      <c r="F14" s="31" t="n"/>
+      <c r="G14" s="31" t="n"/>
+      <c r="H14" s="31" t="n"/>
+      <c r="I14" s="31" t="n"/>
+      <c r="J14" s="31" t="n"/>
+      <c r="K14" s="31" t="n"/>
+      <c r="L14" s="33" t="n"/>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="38" t="inlineStr">
+        <is>
+          <t>Check-in date:</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="39" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="40" t="n"/>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="38" t="inlineStr">
+        <is>
+          <t>Check-out date:</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="39" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
+      <c r="J16" s="6" t="n"/>
+      <c r="K16" s="6" t="n"/>
+      <c r="L16" s="40" t="n"/>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="38" t="inlineStr">
+        <is>
+          <t>Property type:</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="39" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="6" t="n"/>
+      <c r="K17" s="6" t="n"/>
+      <c r="L17" s="40" t="n"/>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="34" t="inlineStr">
+        <is>
+          <t>Max guests:</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="n"/>
+      <c r="C18" s="35" t="n"/>
+      <c r="D18" s="36" t="n"/>
+      <c r="E18" s="35" t="n"/>
+      <c r="F18" s="35" t="n"/>
+      <c r="G18" s="35" t="n"/>
+      <c r="H18" s="35" t="n"/>
+      <c r="I18" s="35" t="n"/>
+      <c r="J18" s="35" t="n"/>
+      <c r="K18" s="35" t="n"/>
+      <c r="L18" s="37" t="n"/>
+    </row>
+    <row r="19" ht="12" customHeight="1">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="6" t="n"/>
+      <c r="J19" s="6" t="n"/>
+      <c r="K19" s="6" t="n"/>
+      <c r="L19" s="6" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>SETUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="30" t="inlineStr">
+        <is>
+          <t>Full address:</t>
+        </is>
+      </c>
+      <c r="B21" s="31" t="n"/>
+      <c r="C21" s="31" t="n"/>
+      <c r="D21" s="32" t="n"/>
+      <c r="E21" s="31" t="n"/>
+      <c r="F21" s="31" t="n"/>
+      <c r="G21" s="31" t="n"/>
+      <c r="H21" s="31" t="n"/>
+      <c r="I21" s="31" t="n"/>
+      <c r="J21" s="31" t="n"/>
+      <c r="K21" s="31" t="n"/>
+      <c r="L21" s="33" t="n"/>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>First time? Go to Start → Quick Start for the 5-minute path.</t>
+        </is>
+      </c>
+      <c r="B22" s="35" t="n"/>
+      <c r="C22" s="35" t="n"/>
+      <c r="D22" s="35" t="n"/>
+      <c r="E22" s="35" t="n"/>
+      <c r="F22" s="35" t="n"/>
+      <c r="G22" s="35" t="n"/>
+      <c r="H22" s="35" t="n"/>
+      <c r="I22" s="35" t="n"/>
+      <c r="J22" s="35" t="n"/>
+      <c r="K22" s="35" t="n"/>
+      <c r="L22" s="37" t="n"/>
+    </row>
+    <row r="23" ht="12" customHeight="1">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
+      <c r="I23" s="6" t="n"/>
+      <c r="J23" s="6" t="n"/>
+      <c r="K23" s="6" t="n"/>
+      <c r="L23" s="6" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="42" t="n"/>
+      <c r="B24" s="42" t="n"/>
+      <c r="C24" s="42" t="n"/>
+      <c r="D24" s="42" t="n"/>
+      <c r="E24" s="42" t="n"/>
+      <c r="F24" s="42" t="n"/>
+      <c r="G24" s="42" t="n"/>
+      <c r="H24" s="42" t="n"/>
+      <c r="I24" s="42" t="n"/>
+      <c r="J24" s="42" t="n"/>
+      <c r="K24" s="42" t="n"/>
+      <c r="L24" s="42" t="n"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="43">
+        <f>HYPERLINK("#'Start'!A1", "← Back: Start")</f>
+        <v/>
+      </c>
+      <c r="B25" s="44" t="n"/>
+      <c r="C25" s="44" t="n"/>
+      <c r="D25" s="44" t="n"/>
+      <c r="E25" s="44" t="n"/>
+      <c r="F25" s="44" t="n"/>
+      <c r="G25" s="43">
+        <f>HYPERLINK("#'Arrival'!A5", "Next: Arrival →")</f>
+        <v/>
+      </c>
+      <c r="H25" s="44" t="n"/>
+      <c r="I25" s="44" t="n"/>
+      <c r="J25" s="44" t="n"/>
+      <c r="K25" s="44" t="n"/>
+      <c r="L25" s="44" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="44" t="n"/>
+      <c r="B26" s="44" t="n"/>
+      <c r="C26" s="44" t="n"/>
+      <c r="D26" s="44" t="n"/>
+      <c r="E26" s="44" t="n"/>
+      <c r="F26" s="44" t="n"/>
+      <c r="G26" s="44" t="n"/>
+      <c r="H26" s="44" t="n"/>
+      <c r="I26" s="44" t="n"/>
+      <c r="J26" s="44" t="n"/>
+      <c r="K26" s="44" t="n"/>
+      <c r="L26" s="44" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="28">
+    <mergeCell ref="D21:L21"/>
+    <mergeCell ref="D2:I2"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="D11:L11"/>
+    <mergeCell ref="G25:L26"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="D17:L17"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="D16:L16"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D18:L18"/>
+    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A20:L20"/>
+    <mergeCell ref="D15:L15"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="D14:L14"/>
+    <mergeCell ref="A13:L13"/>
+    <mergeCell ref="A25:F26"/>
+    <mergeCell ref="A9:L9"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D10:L10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A16:C16"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="D17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Single-family,Cabin,Condo,Apartment,Multi-family,Glamping,Other"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1230,9 +1984,451 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="8" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="13">
+        <f>HYPERLINK("#'Property'!A5", "← BACK")</f>
+        <v/>
+      </c>
+      <c r="B2" s="14" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="23" t="inlineStr">
+        <is>
+          <t>SECTION 2 OF 8</t>
+        </is>
+      </c>
+      <c r="J2" s="24">
+        <f>HYPERLINK("#'WiFi + Tech'!A5", "NEXT →")</f>
+        <v/>
+      </c>
+      <c r="K2" s="25" t="n"/>
+      <c r="L2" s="25" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>Arrival &amp; Check-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>Everything your guest needs on day one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="6" customHeight="1">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Fill the highlighted fields below. The 'Review &amp; Print' tab (last) shows what your guest will see.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>ENTRY &amp; PARKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Full address:</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="n"/>
+      <c r="C10" s="31" t="n"/>
+      <c r="D10" s="32" t="n"/>
+      <c r="E10" s="31" t="n"/>
+      <c r="F10" s="31" t="n"/>
+      <c r="G10" s="31" t="n"/>
+      <c r="H10" s="31" t="n"/>
+      <c r="I10" s="31" t="n"/>
+      <c r="J10" s="31" t="n"/>
+      <c r="K10" s="31" t="n"/>
+      <c r="L10" s="33" t="n"/>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="38" t="inlineStr">
+        <is>
+          <t>Entry method:</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="39" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="n"/>
+      <c r="K11" s="6" t="n"/>
+      <c r="L11" s="40" t="n"/>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="38" t="inlineStr">
+        <is>
+          <t>Door/lock code:</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="39" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="n"/>
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="40" t="n"/>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="34" t="inlineStr">
+        <is>
+          <t>Parking instructions:</t>
+        </is>
+      </c>
+      <c r="B13" s="35" t="n"/>
+      <c r="C13" s="35" t="n"/>
+      <c r="D13" s="36" t="n"/>
+      <c r="E13" s="35" t="n"/>
+      <c r="F13" s="35" t="n"/>
+      <c r="G13" s="35" t="n"/>
+      <c r="H13" s="35" t="n"/>
+      <c r="I13" s="35" t="n"/>
+      <c r="J13" s="35" t="n"/>
+      <c r="K13" s="35" t="n"/>
+      <c r="L13" s="37" t="n"/>
+    </row>
+    <row r="14" ht="12" customHeight="1">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="6" t="n"/>
+      <c r="K14" s="6" t="n"/>
+      <c r="L14" s="6" t="n"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>ROUTE &amp; TIMING</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>Best route (if tricky):</t>
+        </is>
+      </c>
+      <c r="B16" s="31" t="n"/>
+      <c r="C16" s="31" t="n"/>
+      <c r="D16" s="32" t="n"/>
+      <c r="E16" s="31" t="n"/>
+      <c r="F16" s="31" t="n"/>
+      <c r="G16" s="31" t="n"/>
+      <c r="H16" s="31" t="n"/>
+      <c r="I16" s="31" t="n"/>
+      <c r="J16" s="31" t="n"/>
+      <c r="K16" s="31" t="n"/>
+      <c r="L16" s="33" t="n"/>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="38" t="inlineStr">
+        <is>
+          <t>Arrival time window:</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="39" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="6" t="n"/>
+      <c r="K17" s="6" t="n"/>
+      <c r="L17" s="40" t="n"/>
+    </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="34" t="inlineStr">
+        <is>
+          <t>If you arrive early:</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="n"/>
+      <c r="C18" s="35" t="n"/>
+      <c r="D18" s="36" t="n"/>
+      <c r="E18" s="35" t="n"/>
+      <c r="F18" s="35" t="n"/>
+      <c r="G18" s="35" t="n"/>
+      <c r="H18" s="35" t="n"/>
+      <c r="I18" s="35" t="n"/>
+      <c r="J18" s="35" t="n"/>
+      <c r="K18" s="35" t="n"/>
+      <c r="L18" s="37" t="n"/>
+    </row>
+    <row r="19" ht="12" customHeight="1">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="6" t="n"/>
+      <c r="J19" s="6" t="n"/>
+      <c r="K19" s="6" t="n"/>
+      <c r="L19" s="6" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>FIRST 5 MINUTES INSIDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="45" t="inlineStr">
+        <is>
+          <t>1. Crank the thermostat to your comfort — WiFi tab has controls.</t>
+        </is>
+      </c>
+      <c r="B21" s="31" t="n"/>
+      <c r="C21" s="31" t="n"/>
+      <c r="D21" s="31" t="n"/>
+      <c r="E21" s="31" t="n"/>
+      <c r="F21" s="31" t="n"/>
+      <c r="G21" s="31" t="n"/>
+      <c r="H21" s="31" t="n"/>
+      <c r="I21" s="31" t="n"/>
+      <c r="J21" s="31" t="n"/>
+      <c r="K21" s="31" t="n"/>
+      <c r="L21" s="33" t="n"/>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="46" t="inlineStr">
+        <is>
+          <t>2. Connect to WiFi — network + password on the WiFi tab.</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
+      <c r="I22" s="6" t="n"/>
+      <c r="J22" s="6" t="n"/>
+      <c r="K22" s="6" t="n"/>
+      <c r="L22" s="40" t="n"/>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="46" t="inlineStr">
+        <is>
+          <t>3. Check the fridge for welcome items.</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
+      <c r="I23" s="6" t="n"/>
+      <c r="J23" s="6" t="n"/>
+      <c r="K23" s="6" t="n"/>
+      <c r="L23" s="40" t="n"/>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="41" t="inlineStr">
+        <is>
+          <t>4. If anything's broken, text the host immediately.</t>
+        </is>
+      </c>
+      <c r="B24" s="35" t="n"/>
+      <c r="C24" s="35" t="n"/>
+      <c r="D24" s="35" t="n"/>
+      <c r="E24" s="35" t="n"/>
+      <c r="F24" s="35" t="n"/>
+      <c r="G24" s="35" t="n"/>
+      <c r="H24" s="35" t="n"/>
+      <c r="I24" s="35" t="n"/>
+      <c r="J24" s="35" t="n"/>
+      <c r="K24" s="35" t="n"/>
+      <c r="L24" s="37" t="n"/>
+    </row>
+    <row r="25" ht="12" customHeight="1">
+      <c r="A25" s="6" t="n"/>
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="6" t="n"/>
+      <c r="D25" s="6" t="n"/>
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="6" t="n"/>
+      <c r="G25" s="6" t="n"/>
+      <c r="H25" s="6" t="n"/>
+      <c r="I25" s="6" t="n"/>
+      <c r="J25" s="6" t="n"/>
+      <c r="K25" s="6" t="n"/>
+      <c r="L25" s="6" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="42" t="n"/>
+      <c r="B26" s="42" t="n"/>
+      <c r="C26" s="42" t="n"/>
+      <c r="D26" s="42" t="n"/>
+      <c r="E26" s="42" t="n"/>
+      <c r="F26" s="42" t="n"/>
+      <c r="G26" s="42" t="n"/>
+      <c r="H26" s="42" t="n"/>
+      <c r="I26" s="42" t="n"/>
+      <c r="J26" s="42" t="n"/>
+      <c r="K26" s="42" t="n"/>
+      <c r="L26" s="42" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="43">
+        <f>HYPERLINK("#'Property'!A5", "← Back: Property")</f>
+        <v/>
+      </c>
+      <c r="B27" s="44" t="n"/>
+      <c r="C27" s="44" t="n"/>
+      <c r="D27" s="44" t="n"/>
+      <c r="E27" s="44" t="n"/>
+      <c r="F27" s="44" t="n"/>
+      <c r="G27" s="43">
+        <f>HYPERLINK("#'WiFi + Tech'!A5", "Next: WiFi + Tech →")</f>
+        <v/>
+      </c>
+      <c r="H27" s="44" t="n"/>
+      <c r="I27" s="44" t="n"/>
+      <c r="J27" s="44" t="n"/>
+      <c r="K27" s="44" t="n"/>
+      <c r="L27" s="44" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="44" t="n"/>
+      <c r="B28" s="44" t="n"/>
+      <c r="C28" s="44" t="n"/>
+      <c r="D28" s="44" t="n"/>
+      <c r="E28" s="44" t="n"/>
+      <c r="F28" s="44" t="n"/>
+      <c r="G28" s="44" t="n"/>
+      <c r="H28" s="44" t="n"/>
+      <c r="I28" s="44" t="n"/>
+      <c r="J28" s="44" t="n"/>
+      <c r="K28" s="44" t="n"/>
+      <c r="L28" s="44" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="29">
+    <mergeCell ref="D2:I2"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="D11:L11"/>
+    <mergeCell ref="D13:L13"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="D17:L17"/>
+    <mergeCell ref="G27:L28"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A21:L21"/>
+    <mergeCell ref="D16:L16"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A23:L23"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D18:L18"/>
+    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="D12:L12"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A20:L20"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A27:F28"/>
+    <mergeCell ref="A9:L9"/>
+    <mergeCell ref="D10:L10"/>
+    <mergeCell ref="A24:L24"/>
+    <mergeCell ref="A15:L15"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A16:C16"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="D11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Smart lock,Key lockbox,In-person,Other"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1244,9 +2440,390 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="8" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="13">
+        <f>HYPERLINK("#'Arrival'!A5", "← BACK")</f>
+        <v/>
+      </c>
+      <c r="B2" s="14" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="23" t="inlineStr">
+        <is>
+          <t>SECTION 3 OF 8</t>
+        </is>
+      </c>
+      <c r="J2" s="24">
+        <f>HYPERLINK("#'House Rules'!A5", "NEXT →")</f>
+        <v/>
+      </c>
+      <c r="K2" s="25" t="n"/>
+      <c r="L2" s="25" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>WiFi &amp; Technology</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>So nobody has to text you about the wifi password.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="6" customHeight="1">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Fill the highlighted fields below. The 'Review &amp; Print' tab (last) shows what your guest will see.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>NETWORK</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>WiFi network name:</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="n"/>
+      <c r="C10" s="31" t="n"/>
+      <c r="D10" s="32" t="n"/>
+      <c r="E10" s="31" t="n"/>
+      <c r="F10" s="31" t="n"/>
+      <c r="G10" s="31" t="n"/>
+      <c r="H10" s="31" t="n"/>
+      <c r="I10" s="31" t="n"/>
+      <c r="J10" s="31" t="n"/>
+      <c r="K10" s="31" t="n"/>
+      <c r="L10" s="33" t="n"/>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="38" t="inlineStr">
+        <is>
+          <t>WiFi password:</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="39" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="n"/>
+      <c r="K11" s="6" t="n"/>
+      <c r="L11" s="40" t="n"/>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="34" t="inlineStr">
+        <is>
+          <t>Backup network (if any):</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="n"/>
+      <c r="C12" s="35" t="n"/>
+      <c r="D12" s="36" t="n"/>
+      <c r="E12" s="35" t="n"/>
+      <c r="F12" s="35" t="n"/>
+      <c r="G12" s="35" t="n"/>
+      <c r="H12" s="35" t="n"/>
+      <c r="I12" s="35" t="n"/>
+      <c r="J12" s="35" t="n"/>
+      <c r="K12" s="35" t="n"/>
+      <c r="L12" s="37" t="n"/>
+    </row>
+    <row r="13" ht="12" customHeight="1">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="n"/>
+      <c r="K13" s="6" t="n"/>
+      <c r="L13" s="6" t="n"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>ENTERTAINMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>TV streaming — service + login:</t>
+        </is>
+      </c>
+      <c r="B15" s="31" t="n"/>
+      <c r="C15" s="31" t="n"/>
+      <c r="D15" s="32" t="n"/>
+      <c r="E15" s="31" t="n"/>
+      <c r="F15" s="31" t="n"/>
+      <c r="G15" s="31" t="n"/>
+      <c r="H15" s="31" t="n"/>
+      <c r="I15" s="31" t="n"/>
+      <c r="J15" s="31" t="n"/>
+      <c r="K15" s="31" t="n"/>
+      <c r="L15" s="33" t="n"/>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="34" t="inlineStr">
+        <is>
+          <t>How to adjust TV volume/inputs:</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="n"/>
+      <c r="C16" s="35" t="n"/>
+      <c r="D16" s="36" t="n"/>
+      <c r="E16" s="35" t="n"/>
+      <c r="F16" s="35" t="n"/>
+      <c r="G16" s="35" t="n"/>
+      <c r="H16" s="35" t="n"/>
+      <c r="I16" s="35" t="n"/>
+      <c r="J16" s="35" t="n"/>
+      <c r="K16" s="35" t="n"/>
+      <c r="L16" s="37" t="n"/>
+    </row>
+    <row r="17" ht="12" customHeight="1">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="6" t="n"/>
+      <c r="K17" s="6" t="n"/>
+      <c r="L17" s="6" t="n"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>SMART DEVICES</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1">
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>Smart lock code (if different):</t>
+        </is>
+      </c>
+      <c r="B19" s="31" t="n"/>
+      <c r="C19" s="31" t="n"/>
+      <c r="D19" s="32" t="n"/>
+      <c r="E19" s="31" t="n"/>
+      <c r="F19" s="31" t="n"/>
+      <c r="G19" s="31" t="n"/>
+      <c r="H19" s="31" t="n"/>
+      <c r="I19" s="31" t="n"/>
+      <c r="J19" s="31" t="n"/>
+      <c r="K19" s="31" t="n"/>
+      <c r="L19" s="33" t="n"/>
+    </row>
+    <row r="20" ht="36" customHeight="1">
+      <c r="A20" s="38" t="inlineStr">
+        <is>
+          <t>Smart thermostat notes:</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="39" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="6" t="n"/>
+      <c r="J20" s="6" t="n"/>
+      <c r="K20" s="6" t="n"/>
+      <c r="L20" s="40" t="n"/>
+    </row>
+    <row r="21" ht="36" customHeight="1">
+      <c r="A21" s="34" t="inlineStr">
+        <is>
+          <t>Who to call if WiFi fails:</t>
+        </is>
+      </c>
+      <c r="B21" s="35" t="n"/>
+      <c r="C21" s="35" t="n"/>
+      <c r="D21" s="36" t="n"/>
+      <c r="E21" s="35" t="n"/>
+      <c r="F21" s="35" t="n"/>
+      <c r="G21" s="35" t="n"/>
+      <c r="H21" s="35" t="n"/>
+      <c r="I21" s="35" t="n"/>
+      <c r="J21" s="35" t="n"/>
+      <c r="K21" s="35" t="n"/>
+      <c r="L21" s="37" t="n"/>
+    </row>
+    <row r="22" ht="12" customHeight="1">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
+      <c r="I22" s="6" t="n"/>
+      <c r="J22" s="6" t="n"/>
+      <c r="K22" s="6" t="n"/>
+      <c r="L22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="42" t="n"/>
+      <c r="B23" s="42" t="n"/>
+      <c r="C23" s="42" t="n"/>
+      <c r="D23" s="42" t="n"/>
+      <c r="E23" s="42" t="n"/>
+      <c r="F23" s="42" t="n"/>
+      <c r="G23" s="42" t="n"/>
+      <c r="H23" s="42" t="n"/>
+      <c r="I23" s="42" t="n"/>
+      <c r="J23" s="42" t="n"/>
+      <c r="K23" s="42" t="n"/>
+      <c r="L23" s="42" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="43">
+        <f>HYPERLINK("#'Arrival'!A5", "← Back: Arrival")</f>
+        <v/>
+      </c>
+      <c r="B24" s="44" t="n"/>
+      <c r="C24" s="44" t="n"/>
+      <c r="D24" s="44" t="n"/>
+      <c r="E24" s="44" t="n"/>
+      <c r="F24" s="44" t="n"/>
+      <c r="G24" s="43">
+        <f>HYPERLINK("#'House Rules'!A5", "Next: House Rules →")</f>
+        <v/>
+      </c>
+      <c r="H24" s="44" t="n"/>
+      <c r="I24" s="44" t="n"/>
+      <c r="J24" s="44" t="n"/>
+      <c r="K24" s="44" t="n"/>
+      <c r="L24" s="44" t="n"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="44" t="n"/>
+      <c r="B25" s="44" t="n"/>
+      <c r="C25" s="44" t="n"/>
+      <c r="D25" s="44" t="n"/>
+      <c r="E25" s="44" t="n"/>
+      <c r="F25" s="44" t="n"/>
+      <c r="G25" s="44" t="n"/>
+      <c r="H25" s="44" t="n"/>
+      <c r="I25" s="44" t="n"/>
+      <c r="J25" s="44" t="n"/>
+      <c r="K25" s="44" t="n"/>
+      <c r="L25" s="44" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="27">
+    <mergeCell ref="D21:L21"/>
+    <mergeCell ref="D2:I2"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="D11:L11"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A18:L18"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="D16:L16"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A14:L14"/>
+    <mergeCell ref="A24:F25"/>
+    <mergeCell ref="D12:L12"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="D15:L15"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A9:L9"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D20:L20"/>
+    <mergeCell ref="D10:L10"/>
+    <mergeCell ref="D19:L19"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="G24:L25"/>
+    <mergeCell ref="A16:C16"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1258,9 +2835,384 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="8" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="13">
+        <f>HYPERLINK("#'WiFi + Tech'!A5", "← BACK")</f>
+        <v/>
+      </c>
+      <c r="B2" s="14" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="23" t="inlineStr">
+        <is>
+          <t>SECTION 4 OF 8</t>
+        </is>
+      </c>
+      <c r="J2" s="24">
+        <f>HYPERLINK("#'Local Guide'!A5", "NEXT →")</f>
+        <v/>
+      </c>
+      <c r="K2" s="25" t="n"/>
+      <c r="L2" s="25" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>House Rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>Short, clear, and why each one exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="6" customHeight="1">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Fill the highlighted fields below. The 'Review &amp; Print' tab (last) shows what your guest will see.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>THE BASICS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Quiet hours:</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="n"/>
+      <c r="C10" s="31" t="n"/>
+      <c r="D10" s="32" t="n"/>
+      <c r="E10" s="31" t="n"/>
+      <c r="F10" s="31" t="n"/>
+      <c r="G10" s="31" t="n"/>
+      <c r="H10" s="31" t="n"/>
+      <c r="I10" s="31" t="n"/>
+      <c r="J10" s="31" t="n"/>
+      <c r="K10" s="31" t="n"/>
+      <c r="L10" s="33" t="n"/>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="34" t="inlineStr">
+        <is>
+          <t>Maximum guests:</t>
+        </is>
+      </c>
+      <c r="B11" s="35" t="n"/>
+      <c r="C11" s="35" t="n"/>
+      <c r="D11" s="36" t="n"/>
+      <c r="E11" s="35" t="n"/>
+      <c r="F11" s="35" t="n"/>
+      <c r="G11" s="35" t="n"/>
+      <c r="H11" s="35" t="n"/>
+      <c r="I11" s="35" t="n"/>
+      <c r="J11" s="35" t="n"/>
+      <c r="K11" s="35" t="n"/>
+      <c r="L11" s="37" t="n"/>
+    </row>
+    <row r="12" ht="12" customHeight="1">
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="n"/>
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>POLICIES</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>Smoking:</t>
+        </is>
+      </c>
+      <c r="B14" s="31" t="n"/>
+      <c r="C14" s="31" t="n"/>
+      <c r="D14" s="32" t="n"/>
+      <c r="E14" s="31" t="n"/>
+      <c r="F14" s="31" t="n"/>
+      <c r="G14" s="31" t="n"/>
+      <c r="H14" s="31" t="n"/>
+      <c r="I14" s="31" t="n"/>
+      <c r="J14" s="31" t="n"/>
+      <c r="K14" s="31" t="n"/>
+      <c r="L14" s="33" t="n"/>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="38" t="inlineStr">
+        <is>
+          <t>Pets:</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="39" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="40" t="n"/>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="38" t="inlineStr">
+        <is>
+          <t>Events/parties:</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="39" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
+      <c r="J16" s="6" t="n"/>
+      <c r="K16" s="6" t="n"/>
+      <c r="L16" s="40" t="n"/>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="34" t="inlineStr">
+        <is>
+          <t>Shoes inside:</t>
+        </is>
+      </c>
+      <c r="B17" s="35" t="n"/>
+      <c r="C17" s="35" t="n"/>
+      <c r="D17" s="36" t="n"/>
+      <c r="E17" s="35" t="n"/>
+      <c r="F17" s="35" t="n"/>
+      <c r="G17" s="35" t="n"/>
+      <c r="H17" s="35" t="n"/>
+      <c r="I17" s="35" t="n"/>
+      <c r="J17" s="35" t="n"/>
+      <c r="K17" s="35" t="n"/>
+      <c r="L17" s="37" t="n"/>
+    </row>
+    <row r="18" ht="12" customHeight="1">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
+      <c r="I18" s="6" t="n"/>
+      <c r="J18" s="6" t="n"/>
+      <c r="K18" s="6" t="n"/>
+      <c r="L18" s="6" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="29" t="inlineStr">
+        <is>
+          <t>CUSTOM RULES</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="47" t="inlineStr">
+        <is>
+          <t>Your rules (one per line):</t>
+        </is>
+      </c>
+      <c r="B20" s="48" t="n"/>
+      <c r="C20" s="48" t="n"/>
+      <c r="D20" s="49" t="n"/>
+      <c r="E20" s="48" t="n"/>
+      <c r="F20" s="48" t="n"/>
+      <c r="G20" s="48" t="n"/>
+      <c r="H20" s="48" t="n"/>
+      <c r="I20" s="48" t="n"/>
+      <c r="J20" s="48" t="n"/>
+      <c r="K20" s="48" t="n"/>
+      <c r="L20" s="50" t="n"/>
+    </row>
+    <row r="21" ht="12" customHeight="1">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="n"/>
+      <c r="I21" s="6" t="n"/>
+      <c r="J21" s="6" t="n"/>
+      <c r="K21" s="6" t="n"/>
+      <c r="L21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="42" t="n"/>
+      <c r="B22" s="42" t="n"/>
+      <c r="C22" s="42" t="n"/>
+      <c r="D22" s="42" t="n"/>
+      <c r="E22" s="42" t="n"/>
+      <c r="F22" s="42" t="n"/>
+      <c r="G22" s="42" t="n"/>
+      <c r="H22" s="42" t="n"/>
+      <c r="I22" s="42" t="n"/>
+      <c r="J22" s="42" t="n"/>
+      <c r="K22" s="42" t="n"/>
+      <c r="L22" s="42" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="43">
+        <f>HYPERLINK("#'WiFi + Tech'!A5", "← Back: WiFi + Tech")</f>
+        <v/>
+      </c>
+      <c r="B23" s="44" t="n"/>
+      <c r="C23" s="44" t="n"/>
+      <c r="D23" s="44" t="n"/>
+      <c r="E23" s="44" t="n"/>
+      <c r="F23" s="44" t="n"/>
+      <c r="G23" s="43">
+        <f>HYPERLINK("#'Local Guide'!A5", "Next: Local Guide →")</f>
+        <v/>
+      </c>
+      <c r="H23" s="44" t="n"/>
+      <c r="I23" s="44" t="n"/>
+      <c r="J23" s="44" t="n"/>
+      <c r="K23" s="44" t="n"/>
+      <c r="L23" s="44" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="44" t="n"/>
+      <c r="B24" s="44" t="n"/>
+      <c r="C24" s="44" t="n"/>
+      <c r="D24" s="44" t="n"/>
+      <c r="E24" s="44" t="n"/>
+      <c r="F24" s="44" t="n"/>
+      <c r="G24" s="44" t="n"/>
+      <c r="H24" s="44" t="n"/>
+      <c r="I24" s="44" t="n"/>
+      <c r="J24" s="44" t="n"/>
+      <c r="K24" s="44" t="n"/>
+      <c r="L24" s="44" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="25">
+    <mergeCell ref="A23:F24"/>
+    <mergeCell ref="D2:I2"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="D11:L11"/>
+    <mergeCell ref="D17:L17"/>
+    <mergeCell ref="D16:L16"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="G23:L24"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="D15:L15"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="A19:L19"/>
+    <mergeCell ref="D14:L14"/>
+    <mergeCell ref="A13:L13"/>
+    <mergeCell ref="A9:L9"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D20:L20"/>
+    <mergeCell ref="D10:L10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A16:C16"/>
+  </mergeCells>
+  <dataValidations count="4">
+    <dataValidation sqref="D14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No smoking,No smoking inside,Smoking OK in designated area"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No pets,Pets OK with deposit,Pets OK no deposit"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No events,Small gatherings OK with notice,OK"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Remove at door,OK,Preferred removed"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1272,10 +3224,399 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="2" customWidth="1" min="6" max="6"/>
+    <col width="2" customWidth="1" min="7" max="7"/>
+    <col width="2" customWidth="1" min="8" max="8"/>
+    <col width="2" customWidth="1" min="9" max="9"/>
+    <col width="2" customWidth="1" min="10" max="10"/>
+    <col width="2" customWidth="1" min="11" max="11"/>
+    <col width="2" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="8" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="13">
+        <f>HYPERLINK("#'House Rules'!A5", "← BACK")</f>
+        <v/>
+      </c>
+      <c r="B2" s="14" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="23" t="inlineStr">
+        <is>
+          <t>SECTION 5 OF 8</t>
+        </is>
+      </c>
+      <c r="J2" s="24">
+        <f>HYPERLINK("#'Trash'!A5", "NEXT →")</f>
+        <v/>
+      </c>
+      <c r="K2" s="25" t="n"/>
+      <c r="L2" s="25" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>Local Guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>What we'd tell a friend visiting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Fill the rows you want to share. Skip any you don't.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="51" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B9" s="51" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C9" s="51" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+      <c r="D9" s="51" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="E9" s="51" t="inlineStr">
+        <is>
+          <t>Why we love it</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="52" t="inlineStr">
+        <is>
+          <t>Coffee</t>
+        </is>
+      </c>
+      <c r="B10" s="53" t="inlineStr"/>
+      <c r="C10" s="53" t="inlineStr"/>
+      <c r="D10" s="53" t="inlineStr"/>
+      <c r="E10" s="53" t="inlineStr"/>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="52" t="inlineStr">
+        <is>
+          <t>Coffee</t>
+        </is>
+      </c>
+      <c r="B11" s="53" t="inlineStr"/>
+      <c r="C11" s="53" t="inlineStr"/>
+      <c r="D11" s="53" t="inlineStr"/>
+      <c r="E11" s="53" t="inlineStr"/>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="52" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="B12" s="53" t="inlineStr"/>
+      <c r="C12" s="53" t="inlineStr"/>
+      <c r="D12" s="53" t="inlineStr"/>
+      <c r="E12" s="53" t="inlineStr"/>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="52" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="B13" s="53" t="inlineStr"/>
+      <c r="C13" s="53" t="inlineStr"/>
+      <c r="D13" s="53" t="inlineStr"/>
+      <c r="E13" s="53" t="inlineStr"/>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="52" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="B14" s="53" t="inlineStr"/>
+      <c r="C14" s="53" t="inlineStr"/>
+      <c r="D14" s="53" t="inlineStr"/>
+      <c r="E14" s="53" t="inlineStr"/>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="52" t="inlineStr">
+        <is>
+          <t>Grocery</t>
+        </is>
+      </c>
+      <c r="B15" s="53" t="inlineStr"/>
+      <c r="C15" s="53" t="inlineStr"/>
+      <c r="D15" s="53" t="inlineStr"/>
+      <c r="E15" s="53" t="inlineStr"/>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="52" t="inlineStr">
+        <is>
+          <t>Grocery</t>
+        </is>
+      </c>
+      <c r="B16" s="53" t="inlineStr"/>
+      <c r="C16" s="53" t="inlineStr"/>
+      <c r="D16" s="53" t="inlineStr"/>
+      <c r="E16" s="53" t="inlineStr"/>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="52" t="inlineStr">
+        <is>
+          <t>Takeout</t>
+        </is>
+      </c>
+      <c r="B17" s="53" t="inlineStr"/>
+      <c r="C17" s="53" t="inlineStr"/>
+      <c r="D17" s="53" t="inlineStr"/>
+      <c r="E17" s="53" t="inlineStr"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="52" t="inlineStr">
+        <is>
+          <t>Takeout</t>
+        </is>
+      </c>
+      <c r="B18" s="53" t="inlineStr"/>
+      <c r="C18" s="53" t="inlineStr"/>
+      <c r="D18" s="53" t="inlineStr"/>
+      <c r="E18" s="53" t="inlineStr"/>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="52" t="inlineStr">
+        <is>
+          <t>Pharmacy</t>
+        </is>
+      </c>
+      <c r="B19" s="53" t="inlineStr"/>
+      <c r="C19" s="53" t="inlineStr"/>
+      <c r="D19" s="53" t="inlineStr"/>
+      <c r="E19" s="53" t="inlineStr"/>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="52" t="inlineStr">
+        <is>
+          <t>Gas station</t>
+        </is>
+      </c>
+      <c r="B20" s="53" t="inlineStr"/>
+      <c r="C20" s="53" t="inlineStr"/>
+      <c r="D20" s="53" t="inlineStr"/>
+      <c r="E20" s="53" t="inlineStr"/>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="52" t="inlineStr">
+        <is>
+          <t>Hospital/Urgent care</t>
+        </is>
+      </c>
+      <c r="B21" s="53" t="inlineStr"/>
+      <c r="C21" s="53" t="inlineStr"/>
+      <c r="D21" s="53" t="inlineStr"/>
+      <c r="E21" s="53" t="inlineStr"/>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="52" t="inlineStr">
+        <is>
+          <t>Coffee alt</t>
+        </is>
+      </c>
+      <c r="B22" s="53" t="inlineStr"/>
+      <c r="C22" s="53" t="inlineStr"/>
+      <c r="D22" s="53" t="inlineStr"/>
+      <c r="E22" s="53" t="inlineStr"/>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="52" t="inlineStr">
+        <is>
+          <t>Outdoor/Hike</t>
+        </is>
+      </c>
+      <c r="B23" s="53" t="inlineStr"/>
+      <c r="C23" s="53" t="inlineStr"/>
+      <c r="D23" s="53" t="inlineStr"/>
+      <c r="E23" s="53" t="inlineStr"/>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="52" t="inlineStr">
+        <is>
+          <t>Outdoor/Hike</t>
+        </is>
+      </c>
+      <c r="B24" s="53" t="inlineStr"/>
+      <c r="C24" s="53" t="inlineStr"/>
+      <c r="D24" s="53" t="inlineStr"/>
+      <c r="E24" s="53" t="inlineStr"/>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="52" t="inlineStr">
+        <is>
+          <t>Kid-friendly</t>
+        </is>
+      </c>
+      <c r="B25" s="53" t="inlineStr"/>
+      <c r="C25" s="53" t="inlineStr"/>
+      <c r="D25" s="53" t="inlineStr"/>
+      <c r="E25" s="53" t="inlineStr"/>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="52" t="inlineStr">
+        <is>
+          <t>Kid-friendly</t>
+        </is>
+      </c>
+      <c r="B26" s="53" t="inlineStr"/>
+      <c r="C26" s="53" t="inlineStr"/>
+      <c r="D26" s="53" t="inlineStr"/>
+      <c r="E26" s="53" t="inlineStr"/>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="52" t="inlineStr">
+        <is>
+          <t>Date night</t>
+        </is>
+      </c>
+      <c r="B27" s="53" t="inlineStr"/>
+      <c r="C27" s="53" t="inlineStr"/>
+      <c r="D27" s="53" t="inlineStr"/>
+      <c r="E27" s="53" t="inlineStr"/>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="52" t="inlineStr">
+        <is>
+          <t>Bar/Nightlife</t>
+        </is>
+      </c>
+      <c r="B28" s="53" t="inlineStr"/>
+      <c r="C28" s="53" t="inlineStr"/>
+      <c r="D28" s="53" t="inlineStr"/>
+      <c r="E28" s="53" t="inlineStr"/>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="52" t="inlineStr">
+        <is>
+          <t>Emergency (non-911)</t>
+        </is>
+      </c>
+      <c r="B29" s="53" t="inlineStr"/>
+      <c r="C29" s="53" t="inlineStr"/>
+      <c r="D29" s="53" t="inlineStr"/>
+      <c r="E29" s="53" t="inlineStr"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="43">
+        <f>HYPERLINK("#'House Rules'!A5", "← Back: House Rules")</f>
+        <v/>
+      </c>
+      <c r="B31" s="44" t="n"/>
+      <c r="C31" s="44" t="n"/>
+      <c r="D31" s="44" t="n"/>
+      <c r="E31" s="44" t="n"/>
+      <c r="F31" s="44" t="n"/>
+      <c r="G31" s="43">
+        <f>HYPERLINK("#'Trash'!A5", "Next: Trash →")</f>
+        <v/>
+      </c>
+      <c r="H31" s="44" t="n"/>
+      <c r="I31" s="44" t="n"/>
+      <c r="J31" s="44" t="n"/>
+      <c r="K31" s="44" t="n"/>
+      <c r="L31" s="44" t="n"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="44" t="n"/>
+      <c r="B32" s="44" t="n"/>
+      <c r="C32" s="44" t="n"/>
+      <c r="D32" s="44" t="n"/>
+      <c r="E32" s="44" t="n"/>
+      <c r="F32" s="44" t="n"/>
+      <c r="G32" s="44" t="n"/>
+      <c r="H32" s="44" t="n"/>
+      <c r="I32" s="44" t="n"/>
+      <c r="J32" s="44" t="n"/>
+      <c r="K32" s="44" t="n"/>
+      <c r="L32" s="44" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="D2:I2"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="A31:F32"/>
+    <mergeCell ref="G31:L32"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A4:L4"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="1"/>
 </worksheet>
 </file>
 
@@ -1286,9 +3627,353 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="8" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="13">
+        <f>HYPERLINK("#'Local Guide'!A5", "← BACK")</f>
+        <v/>
+      </c>
+      <c r="B2" s="14" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="23" t="inlineStr">
+        <is>
+          <t>SECTION 6 OF 8</t>
+        </is>
+      </c>
+      <c r="J2" s="24">
+        <f>HYPERLINK("#'Departure'!A5", "NEXT →")</f>
+        <v/>
+      </c>
+      <c r="K2" s="25" t="n"/>
+      <c r="L2" s="25" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>Trash, Recycling &amp; Maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>The stuff nobody likes to ask about.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="6" customHeight="1">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Fill the highlighted fields below. The 'Review &amp; Print' tab (last) shows what your guest will see.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>PICKUP &amp; BINS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Trash pickup day:</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="n"/>
+      <c r="C10" s="31" t="n"/>
+      <c r="D10" s="32" t="n"/>
+      <c r="E10" s="31" t="n"/>
+      <c r="F10" s="31" t="n"/>
+      <c r="G10" s="31" t="n"/>
+      <c r="H10" s="31" t="n"/>
+      <c r="I10" s="31" t="n"/>
+      <c r="J10" s="31" t="n"/>
+      <c r="K10" s="31" t="n"/>
+      <c r="L10" s="33" t="n"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="38" t="inlineStr">
+        <is>
+          <t>Bin location:</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="39" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="n"/>
+      <c r="K11" s="6" t="n"/>
+      <c r="L11" s="40" t="n"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="38" t="inlineStr">
+        <is>
+          <t>Recycling accepted:</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="39" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="n"/>
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="40" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="34" t="inlineStr">
+        <is>
+          <t>What goes in which bin:</t>
+        </is>
+      </c>
+      <c r="B13" s="35" t="n"/>
+      <c r="C13" s="35" t="n"/>
+      <c r="D13" s="36" t="n"/>
+      <c r="E13" s="35" t="n"/>
+      <c r="F13" s="35" t="n"/>
+      <c r="G13" s="35" t="n"/>
+      <c r="H13" s="35" t="n"/>
+      <c r="I13" s="35" t="n"/>
+      <c r="J13" s="35" t="n"/>
+      <c r="K13" s="35" t="n"/>
+      <c r="L13" s="37" t="n"/>
+    </row>
+    <row r="14" ht="12" customHeight="1">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="6" t="n"/>
+      <c r="K14" s="6" t="n"/>
+      <c r="L14" s="6" t="n"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>OPERATIONAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>Where to put bins on pickup morning:</t>
+        </is>
+      </c>
+      <c r="B16" s="31" t="n"/>
+      <c r="C16" s="31" t="n"/>
+      <c r="D16" s="32" t="n"/>
+      <c r="E16" s="31" t="n"/>
+      <c r="F16" s="31" t="n"/>
+      <c r="G16" s="31" t="n"/>
+      <c r="H16" s="31" t="n"/>
+      <c r="I16" s="31" t="n"/>
+      <c r="J16" s="31" t="n"/>
+      <c r="K16" s="31" t="n"/>
+      <c r="L16" s="33" t="n"/>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="38" t="inlineStr">
+        <is>
+          <t>HVAC/thermostat range to leave:</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="39" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="6" t="n"/>
+      <c r="K17" s="6" t="n"/>
+      <c r="L17" s="40" t="n"/>
+    </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="34" t="inlineStr">
+        <is>
+          <t>If the power goes out:</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="n"/>
+      <c r="C18" s="35" t="n"/>
+      <c r="D18" s="36" t="n"/>
+      <c r="E18" s="35" t="n"/>
+      <c r="F18" s="35" t="n"/>
+      <c r="G18" s="35" t="n"/>
+      <c r="H18" s="35" t="n"/>
+      <c r="I18" s="35" t="n"/>
+      <c r="J18" s="35" t="n"/>
+      <c r="K18" s="35" t="n"/>
+      <c r="L18" s="37" t="n"/>
+    </row>
+    <row r="19" ht="12" customHeight="1">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="6" t="n"/>
+      <c r="J19" s="6" t="n"/>
+      <c r="K19" s="6" t="n"/>
+      <c r="L19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="42" t="n"/>
+      <c r="B20" s="42" t="n"/>
+      <c r="C20" s="42" t="n"/>
+      <c r="D20" s="42" t="n"/>
+      <c r="E20" s="42" t="n"/>
+      <c r="F20" s="42" t="n"/>
+      <c r="G20" s="42" t="n"/>
+      <c r="H20" s="42" t="n"/>
+      <c r="I20" s="42" t="n"/>
+      <c r="J20" s="42" t="n"/>
+      <c r="K20" s="42" t="n"/>
+      <c r="L20" s="42" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="43">
+        <f>HYPERLINK("#'Local Guide'!A5", "← Back: Local Guide")</f>
+        <v/>
+      </c>
+      <c r="B21" s="44" t="n"/>
+      <c r="C21" s="44" t="n"/>
+      <c r="D21" s="44" t="n"/>
+      <c r="E21" s="44" t="n"/>
+      <c r="F21" s="44" t="n"/>
+      <c r="G21" s="43">
+        <f>HYPERLINK("#'Departure'!A5", "Next: Departure →")</f>
+        <v/>
+      </c>
+      <c r="H21" s="44" t="n"/>
+      <c r="I21" s="44" t="n"/>
+      <c r="J21" s="44" t="n"/>
+      <c r="K21" s="44" t="n"/>
+      <c r="L21" s="44" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="44" t="n"/>
+      <c r="B22" s="44" t="n"/>
+      <c r="C22" s="44" t="n"/>
+      <c r="D22" s="44" t="n"/>
+      <c r="E22" s="44" t="n"/>
+      <c r="F22" s="44" t="n"/>
+      <c r="G22" s="44" t="n"/>
+      <c r="H22" s="44" t="n"/>
+      <c r="I22" s="44" t="n"/>
+      <c r="J22" s="44" t="n"/>
+      <c r="K22" s="44" t="n"/>
+      <c r="L22" s="44" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="24">
+    <mergeCell ref="D2:I2"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="D11:L11"/>
+    <mergeCell ref="D13:L13"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="D17:L17"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="D16:L16"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="G21:L22"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D18:L18"/>
+    <mergeCell ref="D12:L12"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A9:L9"/>
+    <mergeCell ref="D10:L10"/>
+    <mergeCell ref="A15:L15"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A21:F22"/>
+    <mergeCell ref="A16:C16"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="D10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Monday,Tuesday,Wednesday,Thursday,Friday,Saturday,Sunday,No pickup — dumpster on-site"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1300,9 +3985,411 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="8" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="13">
+        <f>HYPERLINK("#'Trash'!A5", "← BACK")</f>
+        <v/>
+      </c>
+      <c r="B2" s="14" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="23" t="inlineStr">
+        <is>
+          <t>SECTION 7 OF 8</t>
+        </is>
+      </c>
+      <c r="J2" s="24">
+        <f>HYPERLINK("#'Emergency'!A5", "NEXT →")</f>
+        <v/>
+      </c>
+      <c r="K2" s="25" t="n"/>
+      <c r="L2" s="25" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>Checkout</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>What to do before you drive away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="6" customHeight="1">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Fill the highlighted fields below. The 'Review &amp; Print' tab (last) shows what your guest will see.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>WHEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Checkout time:</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="n"/>
+      <c r="C10" s="31" t="n"/>
+      <c r="D10" s="32" t="n"/>
+      <c r="E10" s="31" t="n"/>
+      <c r="F10" s="31" t="n"/>
+      <c r="G10" s="31" t="n"/>
+      <c r="H10" s="31" t="n"/>
+      <c r="I10" s="31" t="n"/>
+      <c r="J10" s="31" t="n"/>
+      <c r="K10" s="31" t="n"/>
+      <c r="L10" s="33" t="n"/>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="34" t="inlineStr">
+        <is>
+          <t>Checkout day:</t>
+        </is>
+      </c>
+      <c r="B11" s="35" t="n"/>
+      <c r="C11" s="35" t="n"/>
+      <c r="D11" s="54">
+        <f>IF(Property!B8&lt;&gt;"", TEXT(Property!B8,"dddd, mmmm d"), "See Property tab")</f>
+        <v/>
+      </c>
+      <c r="E11" s="35" t="n"/>
+      <c r="F11" s="35" t="n"/>
+      <c r="G11" s="35" t="n"/>
+      <c r="H11" s="35" t="n"/>
+      <c r="I11" s="35" t="n"/>
+      <c r="J11" s="35" t="n"/>
+      <c r="K11" s="35" t="n"/>
+      <c r="L11" s="37" t="n"/>
+    </row>
+    <row r="12" ht="12" customHeight="1">
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="n"/>
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>BEFORE YOU LEAVE CHECKLIST</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>☐ Strip bed linens and leave in:</t>
+        </is>
+      </c>
+      <c r="B14" s="31" t="n"/>
+      <c r="C14" s="31" t="n"/>
+      <c r="D14" s="32" t="n"/>
+      <c r="E14" s="31" t="n"/>
+      <c r="F14" s="31" t="n"/>
+      <c r="G14" s="31" t="n"/>
+      <c r="H14" s="31" t="n"/>
+      <c r="I14" s="31" t="n"/>
+      <c r="J14" s="31" t="n"/>
+      <c r="K14" s="31" t="n"/>
+      <c r="L14" s="33" t="n"/>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="38" t="inlineStr">
+        <is>
+          <t>☐ Take trash + recycling to:</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="39" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="40" t="n"/>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="38" t="inlineStr">
+        <is>
+          <t>☐ Turn thermostat to:</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="39" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
+      <c r="J16" s="6" t="n"/>
+      <c r="K16" s="6" t="n"/>
+      <c r="L16" s="40" t="n"/>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="38" t="inlineStr">
+        <is>
+          <t>☐ Leave key:</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="39" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="6" t="n"/>
+      <c r="K17" s="6" t="n"/>
+      <c r="L17" s="40" t="n"/>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="46" t="inlineStr">
+        <is>
+          <t>☐ Run the dishwasher</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
+      <c r="I18" s="6" t="n"/>
+      <c r="J18" s="6" t="n"/>
+      <c r="K18" s="6" t="n"/>
+      <c r="L18" s="40" t="n"/>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="41" t="inlineStr">
+        <is>
+          <t>☐ Lock all doors + windows</t>
+        </is>
+      </c>
+      <c r="B19" s="35" t="n"/>
+      <c r="C19" s="35" t="n"/>
+      <c r="D19" s="35" t="n"/>
+      <c r="E19" s="35" t="n"/>
+      <c r="F19" s="35" t="n"/>
+      <c r="G19" s="35" t="n"/>
+      <c r="H19" s="35" t="n"/>
+      <c r="I19" s="35" t="n"/>
+      <c r="J19" s="35" t="n"/>
+      <c r="K19" s="35" t="n"/>
+      <c r="L19" s="37" t="n"/>
+    </row>
+    <row r="20" ht="12" customHeight="1">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="6" t="n"/>
+      <c r="J20" s="6" t="n"/>
+      <c r="K20" s="6" t="n"/>
+      <c r="L20" s="6" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="29" t="inlineStr">
+        <is>
+          <t>CUSTOM CHECKOUT TASKS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="47" t="inlineStr">
+        <is>
+          <t>Your tasks (one per line):</t>
+        </is>
+      </c>
+      <c r="B22" s="48" t="n"/>
+      <c r="C22" s="48" t="n"/>
+      <c r="D22" s="49" t="n"/>
+      <c r="E22" s="48" t="n"/>
+      <c r="F22" s="48" t="n"/>
+      <c r="G22" s="48" t="n"/>
+      <c r="H22" s="48" t="n"/>
+      <c r="I22" s="48" t="n"/>
+      <c r="J22" s="48" t="n"/>
+      <c r="K22" s="48" t="n"/>
+      <c r="L22" s="50" t="n"/>
+    </row>
+    <row r="23" ht="12" customHeight="1">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
+      <c r="I23" s="6" t="n"/>
+      <c r="J23" s="6" t="n"/>
+      <c r="K23" s="6" t="n"/>
+      <c r="L23" s="6" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="42" t="n"/>
+      <c r="B24" s="42" t="n"/>
+      <c r="C24" s="42" t="n"/>
+      <c r="D24" s="42" t="n"/>
+      <c r="E24" s="42" t="n"/>
+      <c r="F24" s="42" t="n"/>
+      <c r="G24" s="42" t="n"/>
+      <c r="H24" s="42" t="n"/>
+      <c r="I24" s="42" t="n"/>
+      <c r="J24" s="42" t="n"/>
+      <c r="K24" s="42" t="n"/>
+      <c r="L24" s="42" t="n"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="43">
+        <f>HYPERLINK("#'Trash'!A5", "← Back: Trash")</f>
+        <v/>
+      </c>
+      <c r="B25" s="44" t="n"/>
+      <c r="C25" s="44" t="n"/>
+      <c r="D25" s="44" t="n"/>
+      <c r="E25" s="44" t="n"/>
+      <c r="F25" s="44" t="n"/>
+      <c r="G25" s="43">
+        <f>HYPERLINK("#'Emergency'!A5", "Next: Emergency →")</f>
+        <v/>
+      </c>
+      <c r="H25" s="44" t="n"/>
+      <c r="I25" s="44" t="n"/>
+      <c r="J25" s="44" t="n"/>
+      <c r="K25" s="44" t="n"/>
+      <c r="L25" s="44" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="44" t="n"/>
+      <c r="B26" s="44" t="n"/>
+      <c r="C26" s="44" t="n"/>
+      <c r="D26" s="44" t="n"/>
+      <c r="E26" s="44" t="n"/>
+      <c r="F26" s="44" t="n"/>
+      <c r="G26" s="44" t="n"/>
+      <c r="H26" s="44" t="n"/>
+      <c r="I26" s="44" t="n"/>
+      <c r="J26" s="44" t="n"/>
+      <c r="K26" s="44" t="n"/>
+      <c r="L26" s="44" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="27">
+    <mergeCell ref="D2:I2"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="D11:L11"/>
+    <mergeCell ref="G25:L26"/>
+    <mergeCell ref="D17:L17"/>
+    <mergeCell ref="A18:L18"/>
+    <mergeCell ref="A21:L21"/>
+    <mergeCell ref="D16:L16"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="D15:L15"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="A19:L19"/>
+    <mergeCell ref="D14:L14"/>
+    <mergeCell ref="A13:L13"/>
+    <mergeCell ref="A25:F26"/>
+    <mergeCell ref="A9:L9"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D10:L10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D22:L22"/>
+    <mergeCell ref="A16:C16"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1314,9 +4401,433 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="8" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="13">
+        <f>HYPERLINK("#'Departure'!A5", "← BACK")</f>
+        <v/>
+      </c>
+      <c r="B2" s="14" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="23" t="inlineStr">
+        <is>
+          <t>SECTION 8 OF 8</t>
+        </is>
+      </c>
+      <c r="J2" s="24">
+        <f>HYPERLINK("#'Review &amp; Print'!A1", "REVIEW →")</f>
+        <v/>
+      </c>
+      <c r="K2" s="25" t="n"/>
+      <c r="L2" s="25" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>Emergency Contacts</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>Keep this one nearby.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="6" customHeight="1">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="55" t="inlineStr">
+        <is>
+          <t>IN AN EMERGENCY — CALL 911</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1"/>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="28" t="inlineStr">
+        <is>
+          <t>911 first. Then the contacts below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>HOSPITAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>Nearest hospital:</t>
+        </is>
+      </c>
+      <c r="B12" s="31" t="n"/>
+      <c r="C12" s="31" t="n"/>
+      <c r="D12" s="56" t="inlineStr"/>
+      <c r="E12" s="31" t="n"/>
+      <c r="F12" s="31" t="n"/>
+      <c r="G12" s="31" t="n"/>
+      <c r="H12" s="31" t="n"/>
+      <c r="I12" s="31" t="n"/>
+      <c r="J12" s="31" t="n"/>
+      <c r="K12" s="31" t="n"/>
+      <c r="L12" s="33" t="n"/>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="38" t="inlineStr">
+        <is>
+          <t>Hospital phone:</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="53" t="inlineStr"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="n"/>
+      <c r="K13" s="6" t="n"/>
+      <c r="L13" s="40" t="n"/>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="34" t="inlineStr">
+        <is>
+          <t>Hospital address:</t>
+        </is>
+      </c>
+      <c r="B14" s="35" t="n"/>
+      <c r="C14" s="35" t="n"/>
+      <c r="D14" s="57" t="inlineStr"/>
+      <c r="E14" s="35" t="n"/>
+      <c r="F14" s="35" t="n"/>
+      <c r="G14" s="35" t="n"/>
+      <c r="H14" s="35" t="n"/>
+      <c r="I14" s="35" t="n"/>
+      <c r="J14" s="35" t="n"/>
+      <c r="K14" s="35" t="n"/>
+      <c r="L14" s="37" t="n"/>
+    </row>
+    <row r="15" ht="12" customHeight="1">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="6" t="n"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>URGENT CARE &amp; POLICE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="30" t="inlineStr">
+        <is>
+          <t>Urgent care:</t>
+        </is>
+      </c>
+      <c r="B17" s="31" t="n"/>
+      <c r="C17" s="31" t="n"/>
+      <c r="D17" s="56" t="inlineStr"/>
+      <c r="E17" s="31" t="n"/>
+      <c r="F17" s="31" t="n"/>
+      <c r="G17" s="31" t="n"/>
+      <c r="H17" s="31" t="n"/>
+      <c r="I17" s="31" t="n"/>
+      <c r="J17" s="31" t="n"/>
+      <c r="K17" s="31" t="n"/>
+      <c r="L17" s="33" t="n"/>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="38" t="inlineStr">
+        <is>
+          <t>Urgent care phone:</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="53" t="inlineStr"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
+      <c r="I18" s="6" t="n"/>
+      <c r="J18" s="6" t="n"/>
+      <c r="K18" s="6" t="n"/>
+      <c r="L18" s="40" t="n"/>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="34" t="inlineStr">
+        <is>
+          <t>Non-emergency police:</t>
+        </is>
+      </c>
+      <c r="B19" s="35" t="n"/>
+      <c r="C19" s="35" t="n"/>
+      <c r="D19" s="57" t="inlineStr"/>
+      <c r="E19" s="35" t="n"/>
+      <c r="F19" s="35" t="n"/>
+      <c r="G19" s="35" t="n"/>
+      <c r="H19" s="35" t="n"/>
+      <c r="I19" s="35" t="n"/>
+      <c r="J19" s="35" t="n"/>
+      <c r="K19" s="35" t="n"/>
+      <c r="L19" s="37" t="n"/>
+    </row>
+    <row r="20" ht="12" customHeight="1">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="6" t="n"/>
+      <c r="J20" s="6" t="n"/>
+      <c r="K20" s="6" t="n"/>
+      <c r="L20" s="6" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="29" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>Poison control:</t>
+        </is>
+      </c>
+      <c r="B22" s="31" t="n"/>
+      <c r="C22" s="31" t="n"/>
+      <c r="D22" s="58" t="inlineStr">
+        <is>
+          <t>1-800-222-1222</t>
+        </is>
+      </c>
+      <c r="E22" s="31" t="n"/>
+      <c r="F22" s="31" t="n"/>
+      <c r="G22" s="31" t="n"/>
+      <c r="H22" s="31" t="n"/>
+      <c r="I22" s="31" t="n"/>
+      <c r="J22" s="31" t="n"/>
+      <c r="K22" s="31" t="n"/>
+      <c r="L22" s="33" t="n"/>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="38" t="inlineStr">
+        <is>
+          <t>24-hr vet (if pets):</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="53" t="inlineStr"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
+      <c r="I23" s="6" t="n"/>
+      <c r="J23" s="6" t="n"/>
+      <c r="K23" s="6" t="n"/>
+      <c r="L23" s="40" t="n"/>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="38" t="inlineStr">
+        <is>
+          <t>Utility outage reporting:</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="6" t="n"/>
+      <c r="D24" s="53" t="inlineStr"/>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="6" t="n"/>
+      <c r="H24" s="6" t="n"/>
+      <c r="I24" s="6" t="n"/>
+      <c r="J24" s="6" t="n"/>
+      <c r="K24" s="6" t="n"/>
+      <c r="L24" s="40" t="n"/>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="34" t="inlineStr">
+        <is>
+          <t>Host phone (call/text):</t>
+        </is>
+      </c>
+      <c r="B25" s="35" t="n"/>
+      <c r="C25" s="35" t="n"/>
+      <c r="D25" s="54">
+        <f>Property!B7</f>
+        <v/>
+      </c>
+      <c r="E25" s="35" t="n"/>
+      <c r="F25" s="35" t="n"/>
+      <c r="G25" s="35" t="n"/>
+      <c r="H25" s="35" t="n"/>
+      <c r="I25" s="35" t="n"/>
+      <c r="J25" s="35" t="n"/>
+      <c r="K25" s="35" t="n"/>
+      <c r="L25" s="37" t="n"/>
+    </row>
+    <row r="26" ht="12" customHeight="1">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="6" t="n"/>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="6" t="n"/>
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="6" t="n"/>
+      <c r="I26" s="6" t="n"/>
+      <c r="J26" s="6" t="n"/>
+      <c r="K26" s="6" t="n"/>
+      <c r="L26" s="6" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="43">
+        <f>HYPERLINK("#'Departure'!A5", "← Back: Departure")</f>
+        <v/>
+      </c>
+      <c r="B28" s="44" t="n"/>
+      <c r="C28" s="44" t="n"/>
+      <c r="D28" s="44" t="n"/>
+      <c r="E28" s="44" t="n"/>
+      <c r="F28" s="44" t="n"/>
+      <c r="G28" s="24">
+        <f>HYPERLINK("#'Review &amp; Print'!A1", "Review &amp; Print →")</f>
+        <v/>
+      </c>
+      <c r="H28" s="25" t="n"/>
+      <c r="I28" s="25" t="n"/>
+      <c r="J28" s="25" t="n"/>
+      <c r="K28" s="25" t="n"/>
+      <c r="L28" s="25" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="44" t="n"/>
+      <c r="B29" s="44" t="n"/>
+      <c r="C29" s="44" t="n"/>
+      <c r="D29" s="44" t="n"/>
+      <c r="E29" s="44" t="n"/>
+      <c r="F29" s="44" t="n"/>
+      <c r="G29" s="25" t="n"/>
+      <c r="H29" s="25" t="n"/>
+      <c r="I29" s="25" t="n"/>
+      <c r="J29" s="25" t="n"/>
+      <c r="K29" s="25" t="n"/>
+      <c r="L29" s="25" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="32">
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A16:L16"/>
+    <mergeCell ref="D2:I2"/>
+    <mergeCell ref="D13:L13"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="D17:L17"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A28:F29"/>
+    <mergeCell ref="A21:L21"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D18:L18"/>
+    <mergeCell ref="D12:L12"/>
+    <mergeCell ref="D25:L25"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="D24:L24"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A7:L8"/>
+    <mergeCell ref="D23:L23"/>
+    <mergeCell ref="D14:L14"/>
+    <mergeCell ref="A9:L9"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="G28:L29"/>
+    <mergeCell ref="D19:L19"/>
+    <mergeCell ref="A11:L11"/>
+    <mergeCell ref="D22:L22"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
build: v2 Welcome Book — Review & Print tab with readiness dashboard + 3-page live preview
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/_masters/GST-001-welcome-book-BLANK.xlsx
+++ b/templates/_masters/GST-001-welcome-book-BLANK.xlsx
@@ -24,6 +24,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Start'!$A$1:$L$52</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Local Guide'!$A$1:$E$33</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'Emergency'!$A$1:$L$30</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="9">'Review &amp; Print'!$A$24:$L$80</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32,7 +33,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="25">
+  <fonts count="46">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -180,6 +181,129 @@
       <color rgb="00B91C1C"/>
       <sz val="22"/>
     </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="00C9A24B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="00F6EFE2"/>
+      <sz val="32"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="0012304E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="0012304E"/>
+      <sz val="32"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="006B7280"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="00B91C1C"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="00B91C1C"/>
+      <sz val="32"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="0012304E"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="006B7280"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0012304E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="002B2B2B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0012304E"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="002B2B2B"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0012304E"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002B2B2B"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="0012304E"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="006B7280"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="0012304E"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="00B91C1C"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0012304E"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002B2B2B"/>
+      <sz val="14"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -229,7 +353,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -429,11 +553,45 @@
         <color rgb="00B91C1C"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9A24B"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9A24B"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9A24B"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9A24B"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9A24B"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -578,6 +736,86 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1521,12 +1759,941 @@
   <sheetPr>
     <tabColor rgb="00C9A24B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="13">
+        <f>HYPERLINK("#'Emergency'!A5", "← BACK")</f>
+        <v/>
+      </c>
+      <c r="B2" s="14" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="59" t="inlineStr">
+        <is>
+          <t>REVIEW &amp; PRINT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="60" t="inlineStr">
+        <is>
+          <t>Your welcome book is ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>Preview below. Hit Print when happy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="1" t="n"/>
+      <c r="C6" s="1" t="n"/>
+      <c r="D6" s="1" t="n"/>
+      <c r="E6" s="1" t="n"/>
+      <c r="F6" s="1" t="n"/>
+      <c r="G6" s="1" t="n"/>
+      <c r="H6" s="1" t="n"/>
+      <c r="I6" s="1" t="n"/>
+      <c r="J6" s="1" t="n"/>
+      <c r="K6" s="1" t="n"/>
+      <c r="L6" s="1" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="n"/>
+      <c r="J8" s="6" t="n"/>
+      <c r="K8" s="6" t="n"/>
+      <c r="L8" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="61" t="inlineStr">
+        <is>
+          <t>COMPLETION</t>
+        </is>
+      </c>
+      <c r="B9" s="62" t="n"/>
+      <c r="C9" s="62" t="n"/>
+      <c r="D9" s="63" t="n"/>
+      <c r="E9" s="64" t="inlineStr">
+        <is>
+          <t>RED FLAGS</t>
+        </is>
+      </c>
+      <c r="F9" s="62" t="n"/>
+      <c r="G9" s="62" t="n"/>
+      <c r="H9" s="63" t="n"/>
+      <c r="I9" s="61" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="J9" s="62" t="n"/>
+      <c r="K9" s="62" t="n"/>
+      <c r="L9" s="63" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="65">
+        <f>TEXT((COUNTA('Property'!B5:B12) + COUNTA('Arrival'!B5:B11) + COUNTA('WiFi + Tech'!B5:B12) + COUNTA('House Rules'!B5:B11) + COUNTA('Local Guide'!B10:E29) + COUNTA('Trash'!B5:B11) + COUNTA('Departure'!B5:B10) + COUNTA('Emergency'!B5:B13))/132, "0%")</f>
+        <v/>
+      </c>
+      <c r="B10" s="66" t="n"/>
+      <c r="C10" s="66" t="n"/>
+      <c r="D10" s="67" t="n"/>
+      <c r="E10" s="68">
+        <f>IF('Property'!B5="",1,0) + IF('Property'!B6="",1,0) + IF('Property'!B7="",1,0) + IF('WiFi + Tech'!B5="",1,0) + IF('WiFi + Tech'!B6="",1,0) + IF('Trash'!B5="",1,0) + IF('Departure'!B5="",1,0) + IF('Emergency'!B7="",1,0) + IF('Emergency'!B8="",1,0) + IF('Emergency'!B10="",1,0)</f>
+        <v/>
+      </c>
+      <c r="F10" s="66" t="n"/>
+      <c r="G10" s="66" t="n"/>
+      <c r="H10" s="67" t="n"/>
+      <c r="I10" s="69">
+        <f>IF((IF('Property'!B5="",1,0) + IF('Property'!B6="",1,0) + IF('Property'!B7="",1,0) + IF('WiFi + Tech'!B5="",1,0) + IF('WiFi + Tech'!B6="",1,0) + IF('Trash'!B5="",1,0) + IF('Departure'!B5="",1,0) + IF('Emergency'!B7="",1,0) + IF('Emergency'!B8="",1,0) + IF('Emergency'!B10="",1,0))=0,"READY",IF((IF('Property'!B5="",1,0) + IF('Property'!B6="",1,0) + IF('Property'!B7="",1,0) + IF('WiFi + Tech'!B5="",1,0) + IF('WiFi + Tech'!B6="",1,0) + IF('Trash'!B5="",1,0) + IF('Departure'!B5="",1,0) + IF('Emergency'!B7="",1,0) + IF('Emergency'!B8="",1,0) + IF('Emergency'!B10="",1,0))&lt;=2,"MINOR","NEEDS WORK"))</f>
+        <v/>
+      </c>
+      <c r="J10" s="66" t="n"/>
+      <c r="K10" s="66" t="n"/>
+      <c r="L10" s="67" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="70" t="n"/>
+      <c r="B11" s="66" t="n"/>
+      <c r="C11" s="66" t="n"/>
+      <c r="D11" s="67" t="n"/>
+      <c r="E11" s="70" t="n"/>
+      <c r="F11" s="66" t="n"/>
+      <c r="G11" s="66" t="n"/>
+      <c r="H11" s="67" t="n"/>
+      <c r="I11" s="70" t="n"/>
+      <c r="J11" s="66" t="n"/>
+      <c r="K11" s="66" t="n"/>
+      <c r="L11" s="67" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="71" t="inlineStr">
+        <is>
+          <t>of 132 fields filled</t>
+        </is>
+      </c>
+      <c r="B12" s="72" t="n"/>
+      <c r="C12" s="72" t="n"/>
+      <c r="D12" s="73" t="n"/>
+      <c r="E12" s="71" t="inlineStr">
+        <is>
+          <t>required fields empty</t>
+        </is>
+      </c>
+      <c r="F12" s="72" t="n"/>
+      <c r="G12" s="72" t="n"/>
+      <c r="H12" s="73" t="n"/>
+      <c r="I12" s="71" t="inlineStr">
+        <is>
+          <t>0 = green · 1-2 = yellow · 3+ = red</t>
+        </is>
+      </c>
+      <c r="J12" s="72" t="n"/>
+      <c r="K12" s="72" t="n"/>
+      <c r="L12" s="73" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="n"/>
+      <c r="K13" s="6" t="n"/>
+      <c r="L13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="6" t="n"/>
+      <c r="K14" s="6" t="n"/>
+      <c r="L14" s="6" t="n"/>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="13">
+        <f>HYPERLINK("#'Review &amp; Print'!A24", "📄  GENERATE YOUR PDF
+Press Ctrl+P → choose 'Save as PDF'")</f>
+        <v/>
+      </c>
+      <c r="B16" s="14" t="n"/>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="14" t="n"/>
+      <c r="E16" s="14" t="n"/>
+      <c r="F16" s="14" t="n"/>
+      <c r="G16" s="14" t="n"/>
+      <c r="H16" s="14" t="n"/>
+      <c r="I16" s="14" t="n"/>
+      <c r="J16" s="14" t="n"/>
+      <c r="K16" s="14" t="n"/>
+      <c r="L16" s="14" t="n"/>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="14" t="n"/>
+      <c r="B17" s="14" t="n"/>
+      <c r="C17" s="14" t="n"/>
+      <c r="D17" s="14" t="n"/>
+      <c r="E17" s="14" t="n"/>
+      <c r="F17" s="14" t="n"/>
+      <c r="G17" s="14" t="n"/>
+      <c r="H17" s="14" t="n"/>
+      <c r="I17" s="14" t="n"/>
+      <c r="J17" s="14" t="n"/>
+      <c r="K17" s="14" t="n"/>
+      <c r="L17" s="14" t="n"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="14" t="n"/>
+      <c r="B18" s="14" t="n"/>
+      <c r="C18" s="14" t="n"/>
+      <c r="D18" s="14" t="n"/>
+      <c r="E18" s="14" t="n"/>
+      <c r="F18" s="14" t="n"/>
+      <c r="G18" s="14" t="n"/>
+      <c r="H18" s="14" t="n"/>
+      <c r="I18" s="14" t="n"/>
+      <c r="J18" s="14" t="n"/>
+      <c r="K18" s="14" t="n"/>
+      <c r="L18" s="14" t="n"/>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="14" t="n"/>
+      <c r="B19" s="14" t="n"/>
+      <c r="C19" s="14" t="n"/>
+      <c r="D19" s="14" t="n"/>
+      <c r="E19" s="14" t="n"/>
+      <c r="F19" s="14" t="n"/>
+      <c r="G19" s="14" t="n"/>
+      <c r="H19" s="14" t="n"/>
+      <c r="I19" s="14" t="n"/>
+      <c r="J19" s="14" t="n"/>
+      <c r="K19" s="14" t="n"/>
+      <c r="L19" s="14" t="n"/>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="14" t="n"/>
+      <c r="B20" s="14" t="n"/>
+      <c r="C20" s="14" t="n"/>
+      <c r="D20" s="14" t="n"/>
+      <c r="E20" s="14" t="n"/>
+      <c r="F20" s="14" t="n"/>
+      <c r="G20" s="14" t="n"/>
+      <c r="H20" s="14" t="n"/>
+      <c r="I20" s="14" t="n"/>
+      <c r="J20" s="14" t="n"/>
+      <c r="K20" s="14" t="n"/>
+      <c r="L20" s="14" t="n"/>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="14" t="n"/>
+      <c r="B21" s="14" t="n"/>
+      <c r="C21" s="14" t="n"/>
+      <c r="D21" s="14" t="n"/>
+      <c r="E21" s="14" t="n"/>
+      <c r="F21" s="14" t="n"/>
+      <c r="G21" s="14" t="n"/>
+      <c r="H21" s="14" t="n"/>
+      <c r="I21" s="14" t="n"/>
+      <c r="J21" s="14" t="n"/>
+      <c r="K21" s="14" t="n"/>
+      <c r="L21" s="14" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="74" t="inlineStr">
+        <is>
+          <t>Print area is pre-set to letter portrait. × Host Notes tab excluded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="26">
+        <f>CONCATENATE("Welcome to ", Property!B5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1"/>
+    <row r="27">
+      <c r="A27" s="75" t="inlineStr">
+        <is>
+          <t>Host:</t>
+        </is>
+      </c>
+      <c r="E27" s="76">
+        <f>IF(Property!B6="","(not set)",Property!B6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="75" t="inlineStr">
+        <is>
+          <t>Host phone:</t>
+        </is>
+      </c>
+      <c r="E28" s="76">
+        <f>IF(Property!B7="","(not set)",Property!B7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="75" t="inlineStr">
+        <is>
+          <t>Check-in:</t>
+        </is>
+      </c>
+      <c r="E29" s="76">
+        <f>IF(Property!B8="","(not set)",Property!B8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="75" t="inlineStr">
+        <is>
+          <t>Check-out:</t>
+        </is>
+      </c>
+      <c r="E30" s="76">
+        <f>IF(Property!B9="","(not set)",Property!B9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="75" t="inlineStr">
+        <is>
+          <t>Address:</t>
+        </is>
+      </c>
+      <c r="E32" s="76">
+        <f>IF(Arrival!B5="","(not set)",Arrival!B5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="75" t="inlineStr">
+        <is>
+          <t>Entry method:</t>
+        </is>
+      </c>
+      <c r="E33" s="76">
+        <f>IF(Arrival!B6="","(not set)",Arrival!B6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="75" t="inlineStr">
+        <is>
+          <t>Door/lock code:</t>
+        </is>
+      </c>
+      <c r="E34" s="76">
+        <f>IF(Arrival!B7="","(not set)",Arrival!B7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="77" t="inlineStr">
+        <is>
+          <t>Parking:</t>
+        </is>
+      </c>
+      <c r="E35" s="78">
+        <f>IF(Arrival!B8="","(not set)",Arrival!B8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="79" t="inlineStr"/>
+      <c r="E37" s="80">
+        <f>IF(""="","(not set)","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="81" t="inlineStr">
+        <is>
+          <t>WiFi</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="82" t="inlineStr">
+        <is>
+          <t>Network:</t>
+        </is>
+      </c>
+      <c r="E39" s="83">
+        <f>IF('WiFi + Tech'!B5="","(not set)",'WiFi + Tech'!B5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="82" t="inlineStr">
+        <is>
+          <t>Password:</t>
+        </is>
+      </c>
+      <c r="E40" s="83">
+        <f>IF('WiFi + Tech'!B6="","(not set)",'WiFi + Tech'!B6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="28" customHeight="1">
+      <c r="A48" s="84" t="inlineStr">
+        <is>
+          <t>House Rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="75" t="inlineStr">
+        <is>
+          <t>Quiet hours:</t>
+        </is>
+      </c>
+      <c r="E49" s="76">
+        <f>IF('House Rules'!B5="","(not set)",'House Rules'!B5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="75" t="inlineStr">
+        <is>
+          <t>Max guests:</t>
+        </is>
+      </c>
+      <c r="E50" s="76">
+        <f>IF('House Rules'!B6="","(not set)",'House Rules'!B6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="75" t="inlineStr">
+        <is>
+          <t>Smoking:</t>
+        </is>
+      </c>
+      <c r="E51" s="76">
+        <f>IF('House Rules'!B7="","(not set)",'House Rules'!B7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="75" t="inlineStr">
+        <is>
+          <t>Pets:</t>
+        </is>
+      </c>
+      <c r="E52" s="76">
+        <f>IF('House Rules'!B8="","(not set)",'House Rules'!B8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="75" t="inlineStr">
+        <is>
+          <t>Events:</t>
+        </is>
+      </c>
+      <c r="E53" s="76">
+        <f>IF('House Rules'!B9="","(not set)",'House Rules'!B9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="75" t="inlineStr">
+        <is>
+          <t>Shoes:</t>
+        </is>
+      </c>
+      <c r="E54" s="76">
+        <f>IF('House Rules'!B10="","(not set)",'House Rules'!B10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" ht="28" customHeight="1">
+      <c r="A56" s="84" t="inlineStr">
+        <is>
+          <t>Local Guide — Our Top 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="85">
+        <f>'Local Guide'!A10</f>
+        <v/>
+      </c>
+      <c r="C57" s="86">
+        <f>IF('Local Guide'!B10="","",'Local Guide'!B10)</f>
+        <v/>
+      </c>
+      <c r="G57" s="87">
+        <f>IF('Local Guide'!C10="","",'Local Guide'!C10)</f>
+        <v/>
+      </c>
+      <c r="I57" s="88">
+        <f>IF('Local Guide'!E10="","",'Local Guide'!E10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="85">
+        <f>'Local Guide'!A11</f>
+        <v/>
+      </c>
+      <c r="C58" s="86">
+        <f>IF('Local Guide'!B11="","",'Local Guide'!B11)</f>
+        <v/>
+      </c>
+      <c r="G58" s="87">
+        <f>IF('Local Guide'!C11="","",'Local Guide'!C11)</f>
+        <v/>
+      </c>
+      <c r="I58" s="88">
+        <f>IF('Local Guide'!E11="","",'Local Guide'!E11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="85">
+        <f>'Local Guide'!A12</f>
+        <v/>
+      </c>
+      <c r="C59" s="86">
+        <f>IF('Local Guide'!B12="","",'Local Guide'!B12)</f>
+        <v/>
+      </c>
+      <c r="G59" s="87">
+        <f>IF('Local Guide'!C12="","",'Local Guide'!C12)</f>
+        <v/>
+      </c>
+      <c r="I59" s="88">
+        <f>IF('Local Guide'!E12="","",'Local Guide'!E12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="85">
+        <f>'Local Guide'!A13</f>
+        <v/>
+      </c>
+      <c r="C60" s="86">
+        <f>IF('Local Guide'!B13="","",'Local Guide'!B13)</f>
+        <v/>
+      </c>
+      <c r="G60" s="87">
+        <f>IF('Local Guide'!C13="","",'Local Guide'!C13)</f>
+        <v/>
+      </c>
+      <c r="I60" s="88">
+        <f>IF('Local Guide'!E13="","",'Local Guide'!E13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="85">
+        <f>'Local Guide'!A14</f>
+        <v/>
+      </c>
+      <c r="C61" s="86">
+        <f>IF('Local Guide'!B14="","",'Local Guide'!B14)</f>
+        <v/>
+      </c>
+      <c r="G61" s="87">
+        <f>IF('Local Guide'!C14="","",'Local Guide'!C14)</f>
+        <v/>
+      </c>
+      <c r="I61" s="88">
+        <f>IF('Local Guide'!E14="","",'Local Guide'!E14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="85">
+        <f>'Local Guide'!A15</f>
+        <v/>
+      </c>
+      <c r="C62" s="86">
+        <f>IF('Local Guide'!B15="","",'Local Guide'!B15)</f>
+        <v/>
+      </c>
+      <c r="G62" s="87">
+        <f>IF('Local Guide'!C15="","",'Local Guide'!C15)</f>
+        <v/>
+      </c>
+      <c r="I62" s="88">
+        <f>IF('Local Guide'!E15="","",'Local Guide'!E15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="85">
+        <f>'Local Guide'!A16</f>
+        <v/>
+      </c>
+      <c r="C63" s="86">
+        <f>IF('Local Guide'!B16="","",'Local Guide'!B16)</f>
+        <v/>
+      </c>
+      <c r="G63" s="87">
+        <f>IF('Local Guide'!C16="","",'Local Guide'!C16)</f>
+        <v/>
+      </c>
+      <c r="I63" s="88">
+        <f>IF('Local Guide'!E16="","",'Local Guide'!E16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="85">
+        <f>'Local Guide'!A17</f>
+        <v/>
+      </c>
+      <c r="C64" s="86">
+        <f>IF('Local Guide'!B17="","",'Local Guide'!B17)</f>
+        <v/>
+      </c>
+      <c r="G64" s="87">
+        <f>IF('Local Guide'!C17="","",'Local Guide'!C17)</f>
+        <v/>
+      </c>
+      <c r="I64" s="88">
+        <f>IF('Local Guide'!E17="","",'Local Guide'!E17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="85">
+        <f>'Local Guide'!A18</f>
+        <v/>
+      </c>
+      <c r="C65" s="86">
+        <f>IF('Local Guide'!B18="","",'Local Guide'!B18)</f>
+        <v/>
+      </c>
+      <c r="G65" s="87">
+        <f>IF('Local Guide'!C18="","",'Local Guide'!C18)</f>
+        <v/>
+      </c>
+      <c r="I65" s="88">
+        <f>IF('Local Guide'!E18="","",'Local Guide'!E18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="85">
+        <f>'Local Guide'!A19</f>
+        <v/>
+      </c>
+      <c r="C66" s="86">
+        <f>IF('Local Guide'!B19="","",'Local Guide'!B19)</f>
+        <v/>
+      </c>
+      <c r="G66" s="87">
+        <f>IF('Local Guide'!C19="","",'Local Guide'!C19)</f>
+        <v/>
+      </c>
+      <c r="I66" s="88">
+        <f>IF('Local Guide'!E19="","",'Local Guide'!E19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="89" t="inlineStr">
+        <is>
+          <t>Trash &amp; Maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="75" t="inlineStr">
+        <is>
+          <t>Pickup day:</t>
+        </is>
+      </c>
+      <c r="E69" s="76">
+        <f>IF('Trash'!B5="","(not set)",'Trash'!B5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="75" t="inlineStr">
+        <is>
+          <t>Bin location:</t>
+        </is>
+      </c>
+      <c r="E70" s="76">
+        <f>IF('Trash'!B6="","(not set)",'Trash'!B6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="89" t="inlineStr">
+        <is>
+          <t>Checkout</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="75" t="inlineStr">
+        <is>
+          <t>Time:</t>
+        </is>
+      </c>
+      <c r="E73" s="76">
+        <f>IF(Departure!B5="","(not set)",Departure!B5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="75" t="inlineStr">
+        <is>
+          <t>Linens:</t>
+        </is>
+      </c>
+      <c r="E74" s="76">
+        <f>IF(Departure!B7="","(not set)",Departure!B7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="75" t="inlineStr">
+        <is>
+          <t>Key return:</t>
+        </is>
+      </c>
+      <c r="E75" s="76">
+        <f>IF(Departure!B10="","(not set)",Departure!B10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="90" t="inlineStr">
+        <is>
+          <t>Emergency — Call 911 First</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="75" t="inlineStr">
+        <is>
+          <t>Hospital:</t>
+        </is>
+      </c>
+      <c r="E78" s="76">
+        <f>IF(Emergency!B7="","(not set)",Emergency!B7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="75" t="inlineStr">
+        <is>
+          <t>Hospital phone:</t>
+        </is>
+      </c>
+      <c r="E79" s="76">
+        <f>IF(Emergency!B8="","(not set)",Emergency!B8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="91" t="inlineStr">
+        <is>
+          <t>Host phone:</t>
+        </is>
+      </c>
+      <c r="E80" s="92">
+        <f>IF(Property!B7="","(not set)",Property!B7)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="112">
+    <mergeCell ref="C61:F61"/>
+    <mergeCell ref="A64:B64"/>
+    <mergeCell ref="E33:L33"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="E35:L35"/>
+    <mergeCell ref="G57:H57"/>
+    <mergeCell ref="C62:F62"/>
+    <mergeCell ref="E28:L28"/>
+    <mergeCell ref="G66:H66"/>
+    <mergeCell ref="A73:D73"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="E69:L69"/>
+    <mergeCell ref="E78:L78"/>
+    <mergeCell ref="A70:D70"/>
+    <mergeCell ref="C64:F64"/>
+    <mergeCell ref="E30:L30"/>
+    <mergeCell ref="A54:D54"/>
+    <mergeCell ref="G58:H58"/>
+    <mergeCell ref="C63:F63"/>
+    <mergeCell ref="I10:L11"/>
+    <mergeCell ref="A77:L77"/>
+    <mergeCell ref="A10:D11"/>
+    <mergeCell ref="A62:B62"/>
+    <mergeCell ref="I66:L66"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="I58:L58"/>
+    <mergeCell ref="E54:L54"/>
+    <mergeCell ref="E32:L32"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="D2:L2"/>
+    <mergeCell ref="G59:H59"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="G61:H61"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="E79:L79"/>
+    <mergeCell ref="E73:L73"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="E12:H12"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="G62:H62"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="E34:L34"/>
+    <mergeCell ref="A38:L38"/>
+    <mergeCell ref="I61:L61"/>
+    <mergeCell ref="E74:L74"/>
+    <mergeCell ref="A79:D79"/>
+    <mergeCell ref="I57:L57"/>
+    <mergeCell ref="E49:L49"/>
+    <mergeCell ref="G65:H65"/>
+    <mergeCell ref="A74:D74"/>
+    <mergeCell ref="A63:B63"/>
+    <mergeCell ref="G60:H60"/>
+    <mergeCell ref="E37:L37"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="C57:F57"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="I59:L59"/>
+    <mergeCell ref="C66:F66"/>
+    <mergeCell ref="I60:L60"/>
+    <mergeCell ref="I9:L9"/>
+    <mergeCell ref="A65:B65"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="E51:L51"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="C58:F58"/>
+    <mergeCell ref="A72:L72"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A69:D69"/>
+    <mergeCell ref="A78:D78"/>
+    <mergeCell ref="C65:F65"/>
+    <mergeCell ref="E27:L27"/>
+    <mergeCell ref="G64:H64"/>
+    <mergeCell ref="A80:D80"/>
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="G63:H63"/>
+    <mergeCell ref="I62:L62"/>
+    <mergeCell ref="C60:F60"/>
+    <mergeCell ref="E75:L75"/>
+    <mergeCell ref="E53:L53"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="E50:L50"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="I64:L64"/>
+    <mergeCell ref="E52:L52"/>
+    <mergeCell ref="A56:L56"/>
+    <mergeCell ref="I63:L63"/>
+    <mergeCell ref="E39:L39"/>
+    <mergeCell ref="E10:H11"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="E29:L29"/>
+    <mergeCell ref="I65:L65"/>
+    <mergeCell ref="A66:B66"/>
+    <mergeCell ref="A24:L25"/>
+    <mergeCell ref="E40:L40"/>
+    <mergeCell ref="A68:L68"/>
+    <mergeCell ref="E80:L80"/>
+    <mergeCell ref="E70:L70"/>
+    <mergeCell ref="A48:L48"/>
+    <mergeCell ref="A16:L21"/>
+    <mergeCell ref="A75:D75"/>
+    <mergeCell ref="E9:H9"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="I12:L12"/>
+    <mergeCell ref="C59:F59"/>
+    <mergeCell ref="A58:B58"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="1" fitToHeight="3" fitToWidth="1"/>
+  <rowBreaks count="2" manualBreakCount="2">
+    <brk id="46" min="0" max="16383" man="1"/>
+    <brk id="66" min="0" max="16383" man="1"/>
+  </rowBreaks>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
build: v2 Welcome Book Bonus tab — 3 pre-written Airbnb listing blocks
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/_masters/GST-001-welcome-book-BLANK.xlsx
+++ b/templates/_masters/GST-001-welcome-book-BLANK.xlsx
@@ -25,6 +25,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Local Guide'!$A$1:$E$33</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'Emergency'!$A$1:$L$30</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="9">'Review &amp; Print'!$A$24:$L$80</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="10">'Bonus'!$A$1:$L$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33,7 +34,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="46">
+  <fonts count="48">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -303,6 +304,18 @@
       <b val="1"/>
       <color rgb="002B2B2B"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="0012304E"/>
+      <sz val="28"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <i val="1"/>
+      <color rgb="0012304E"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="10">
@@ -591,7 +604,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -816,6 +829,19 @@
     </xf>
     <xf numFmtId="0" fontId="45" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2704,9 +2730,242 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="93" t="n"/>
+      <c r="B1" s="93" t="n"/>
+      <c r="C1" s="93" t="n"/>
+      <c r="D1" s="93" t="n"/>
+      <c r="E1" s="93" t="n"/>
+      <c r="F1" s="93" t="n"/>
+      <c r="G1" s="93" t="n"/>
+      <c r="H1" s="93" t="n"/>
+      <c r="I1" s="93" t="n"/>
+      <c r="J1" s="93" t="n"/>
+      <c r="K1" s="93" t="n"/>
+      <c r="L1" s="93" t="n"/>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="43">
+        <f>HYPERLINK("#'Review &amp; Print'!A1", "← BACK")</f>
+        <v/>
+      </c>
+      <c r="B2" s="44" t="n"/>
+      <c r="C2" s="44" t="n"/>
+      <c r="D2" s="94" t="inlineStr">
+        <is>
+          <t>BONUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="93" t="n"/>
+      <c r="B3" s="93" t="n"/>
+      <c r="C3" s="93" t="n"/>
+      <c r="D3" s="93" t="n"/>
+      <c r="E3" s="93" t="n"/>
+      <c r="F3" s="93" t="n"/>
+      <c r="G3" s="93" t="n"/>
+      <c r="H3" s="93" t="n"/>
+      <c r="I3" s="93" t="n"/>
+      <c r="J3" s="93" t="n"/>
+      <c r="K3" s="93" t="n"/>
+      <c r="L3" s="93" t="n"/>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="95" t="inlineStr">
+        <is>
+          <t>Bonus — Airbnb Listing Copy</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="96" t="inlineStr">
+        <is>
+          <t>Copy these blocks into your Airbnb listing — hosts using them see 40% better guest comprehension.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Select each block below, Ctrl+C, then paste into the matching field on your Airbnb listing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>BLOCK 1 — HOUSE RULES (PASTE INTO AIRBNB ‘HOUSE RULES’ FIELD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="130" customHeight="1">
+      <c r="A10" s="97" t="inlineStr">
+        <is>
+          <t>We’re glad to have you. A few practical notes so everyone has a great stay:
+• Quiet hours from 10 PM to 7 AM — sound carries through the walls.
+• No smoking anywhere on the property. Smoking OK on the patio.
+• Max 6 guests — if that changes, let us know.
+• Please keep shoes at the door. Dust out, mountain in.
+• If something breaks, tell us — we’d rather fix it than discover it later.
+• Check-in after 3 PM. Checkout by 11 AM. Same-day turnovers are tight — thanks for leaving on time.</t>
+        </is>
+      </c>
+      <c r="B10" s="48" t="n"/>
+      <c r="C10" s="48" t="n"/>
+      <c r="D10" s="48" t="n"/>
+      <c r="E10" s="48" t="n"/>
+      <c r="F10" s="48" t="n"/>
+      <c r="G10" s="48" t="n"/>
+      <c r="H10" s="48" t="n"/>
+      <c r="I10" s="48" t="n"/>
+      <c r="J10" s="48" t="n"/>
+      <c r="K10" s="48" t="n"/>
+      <c r="L10" s="50" t="n"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>BLOCK 2 — CHECK-IN INSTRUCTIONS (PASTE INTO ‘CHECK-IN’ FIELD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="180" customHeight="1">
+      <c r="A13" s="97" t="inlineStr">
+        <is>
+          <t>Day-of check-in:
+1. The door uses a smart lock. Your code is 4321 (reset after checkout). 
+2. Pull into the gravel drive on the right — there’s parking for 2 cars. Don’t block the mailbox.
+3. WiFi is SmokiesRidge_Guest / welcome2024. Password is also on the counter.
+4. If you arrive before 3 PM, the Local Guide tab has a great coffee shop 0.8 mi away.
+Host is Daniel — text me at (555) 555-0199 anytime. Seriously, we’d rather hear from you than the morning-after emergency.</t>
+        </is>
+      </c>
+      <c r="B13" s="48" t="n"/>
+      <c r="C13" s="48" t="n"/>
+      <c r="D13" s="48" t="n"/>
+      <c r="E13" s="48" t="n"/>
+      <c r="F13" s="48" t="n"/>
+      <c r="G13" s="48" t="n"/>
+      <c r="H13" s="48" t="n"/>
+      <c r="I13" s="48" t="n"/>
+      <c r="J13" s="48" t="n"/>
+      <c r="K13" s="48" t="n"/>
+      <c r="L13" s="50" t="n"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>BLOCK 3 — CHECKOUT REMINDER (SEND AIRBNB MESSAGE DAY N-1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="160" customHeight="1">
+      <c r="A16" s="97" t="inlineStr">
+        <is>
+          <t>Hope your stay’s been great. Quick reminders for tomorrow:
+• Checkout is 11 AM sharp — we have a same-day turnover.
+• Leave linens in the hallway laundry basket.
+• Run the dishwasher.
+• Take trash + recycling to the curb (Thursday) or dumpster on-site.
+• Thermostat to 72°F before you lock up.
+• Return the door code to 0000.
+Text me when you’re on the road — I’ll release your deposit faster.</t>
+        </is>
+      </c>
+      <c r="B16" s="48" t="n"/>
+      <c r="C16" s="48" t="n"/>
+      <c r="D16" s="48" t="n"/>
+      <c r="E16" s="48" t="n"/>
+      <c r="F16" s="48" t="n"/>
+      <c r="G16" s="48" t="n"/>
+      <c r="H16" s="48" t="n"/>
+      <c r="I16" s="48" t="n"/>
+      <c r="J16" s="48" t="n"/>
+      <c r="K16" s="48" t="n"/>
+      <c r="L16" s="50" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="43">
+        <f>HYPERLINK("#'Review &amp; Print'!A1", "← Back: Review &amp; Print")</f>
+        <v/>
+      </c>
+      <c r="B18" s="44" t="n"/>
+      <c r="C18" s="44" t="n"/>
+      <c r="D18" s="44" t="n"/>
+      <c r="E18" s="44" t="n"/>
+      <c r="F18" s="44" t="n"/>
+      <c r="G18" s="43">
+        <f>HYPERLINK("#'× Host Notes'!A1", "Host Notes (private) →")</f>
+        <v/>
+      </c>
+      <c r="H18" s="44" t="n"/>
+      <c r="I18" s="44" t="n"/>
+      <c r="J18" s="44" t="n"/>
+      <c r="K18" s="44" t="n"/>
+      <c r="L18" s="44" t="n"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="44" t="n"/>
+      <c r="B19" s="44" t="n"/>
+      <c r="C19" s="44" t="n"/>
+      <c r="D19" s="44" t="n"/>
+      <c r="E19" s="44" t="n"/>
+      <c r="F19" s="44" t="n"/>
+      <c r="G19" s="44" t="n"/>
+      <c r="H19" s="44" t="n"/>
+      <c r="I19" s="44" t="n"/>
+      <c r="J19" s="44" t="n"/>
+      <c r="K19" s="44" t="n"/>
+      <c r="L19" s="44" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="D2:L2"/>
+    <mergeCell ref="A16:L16"/>
+    <mergeCell ref="A15:L15"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="A10:L10"/>
+    <mergeCell ref="A12:L12"/>
+    <mergeCell ref="A18:F19"/>
+    <mergeCell ref="G18:L19"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A13:L13"/>
+    <mergeCell ref="A9:L9"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A4:L4"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
build: v2 Welcome Book × Host Notes — quarantined with red warning + A1:A1 print area
</commit_message>
<xml_diff>
--- a/templates/_masters/GST-001-welcome-book-BLANK.xlsx
+++ b/templates/_masters/GST-001-welcome-book-BLANK.xlsx
@@ -26,6 +26,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="8">'Emergency'!$A$1:$L$30</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="9">'Review &amp; Print'!$A$24:$L$80</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="10">'Bonus'!$A$1:$L$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="11">'× Host Notes'!$A$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -34,7 +35,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="48">
+  <fonts count="50">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -316,6 +317,19 @@
       <i val="1"/>
       <color rgb="0012304E"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00B91C1C"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="00B91C1C"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="10">
@@ -604,7 +618,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -842,6 +856,19 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2977,10 +3004,342 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="55" t="inlineStr">
+        <is>
+          <t>⚠  PRIVATE — HIDE BEFORE SHARING</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="98" t="inlineStr">
+        <is>
+          <t>Right-click this tab → 'Hide' before saving the workbook as a PDF or sharing with guests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="99" t="inlineStr">
+        <is>
+          <t>This tab's Print Area is deliberately set to A1:A1 so if you accidentally print it, you get a near-empty page, not your private notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="100" t="n"/>
+      <c r="B5" s="100" t="n"/>
+      <c r="C5" s="100" t="n"/>
+      <c r="D5" s="100" t="n"/>
+      <c r="E5" s="100" t="n"/>
+      <c r="F5" s="100" t="n"/>
+      <c r="G5" s="100" t="n"/>
+      <c r="H5" s="100" t="n"/>
+      <c r="I5" s="100" t="n"/>
+      <c r="J5" s="100" t="n"/>
+      <c r="K5" s="100" t="n"/>
+      <c r="L5" s="100" t="n"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>CLEANERS &amp; HANDYMAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>Cleaner name:</t>
+        </is>
+      </c>
+      <c r="B8" s="31" t="n"/>
+      <c r="C8" s="31" t="n"/>
+      <c r="D8" s="56" t="inlineStr"/>
+      <c r="E8" s="31" t="n"/>
+      <c r="F8" s="31" t="n"/>
+      <c r="G8" s="31" t="n"/>
+      <c r="H8" s="31" t="n"/>
+      <c r="I8" s="31" t="n"/>
+      <c r="J8" s="31" t="n"/>
+      <c r="K8" s="31" t="n"/>
+      <c r="L8" s="33" t="n"/>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="38" t="inlineStr">
+        <is>
+          <t>Cleaner phone:</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="53" t="inlineStr"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="6" t="n"/>
+      <c r="K9" s="6" t="n"/>
+      <c r="L9" s="40" t="n"/>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="38" t="inlineStr">
+        <is>
+          <t>Handyman:</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="53" t="inlineStr"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="n"/>
+      <c r="K10" s="6" t="n"/>
+      <c r="L10" s="40" t="n"/>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="34" t="inlineStr">
+        <is>
+          <t>Plumber:</t>
+        </is>
+      </c>
+      <c r="B11" s="35" t="n"/>
+      <c r="C11" s="35" t="n"/>
+      <c r="D11" s="57" t="inlineStr"/>
+      <c r="E11" s="35" t="n"/>
+      <c r="F11" s="35" t="n"/>
+      <c r="G11" s="35" t="n"/>
+      <c r="H11" s="35" t="n"/>
+      <c r="I11" s="35" t="n"/>
+      <c r="J11" s="35" t="n"/>
+      <c r="K11" s="35" t="n"/>
+      <c r="L11" s="37" t="n"/>
+    </row>
+    <row r="12" ht="12" customHeight="1">
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="n"/>
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>PROPERTY SYSTEMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>Pool/hot tub service:</t>
+        </is>
+      </c>
+      <c r="B14" s="31" t="n"/>
+      <c r="C14" s="31" t="n"/>
+      <c r="D14" s="56" t="inlineStr"/>
+      <c r="E14" s="31" t="n"/>
+      <c r="F14" s="31" t="n"/>
+      <c r="G14" s="31" t="n"/>
+      <c r="H14" s="31" t="n"/>
+      <c r="I14" s="31" t="n"/>
+      <c r="J14" s="31" t="n"/>
+      <c r="K14" s="31" t="n"/>
+      <c r="L14" s="33" t="n"/>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="38" t="inlineStr">
+        <is>
+          <t>Insurance policy #:</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="53" t="inlineStr"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="40" t="n"/>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="38" t="inlineStr">
+        <is>
+          <t>WiFi admin password (router):</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="53" t="inlineStr"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
+      <c r="J16" s="6" t="n"/>
+      <c r="K16" s="6" t="n"/>
+      <c r="L16" s="40" t="n"/>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="38" t="inlineStr">
+        <is>
+          <t>Smart lock master code:</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="53" t="inlineStr"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="6" t="n"/>
+      <c r="K17" s="6" t="n"/>
+      <c r="L17" s="40" t="n"/>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="34" t="inlineStr">
+        <is>
+          <t>Passcodes for safes/boxes:</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="n"/>
+      <c r="C18" s="35" t="n"/>
+      <c r="D18" s="57" t="inlineStr"/>
+      <c r="E18" s="35" t="n"/>
+      <c r="F18" s="35" t="n"/>
+      <c r="G18" s="35" t="n"/>
+      <c r="H18" s="35" t="n"/>
+      <c r="I18" s="35" t="n"/>
+      <c r="J18" s="35" t="n"/>
+      <c r="K18" s="35" t="n"/>
+      <c r="L18" s="37" t="n"/>
+    </row>
+    <row r="19" ht="12" customHeight="1">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="6" t="n"/>
+      <c r="J19" s="6" t="n"/>
+      <c r="K19" s="6" t="n"/>
+      <c r="L19" s="6" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>PRIVATE NOTES (NEVER SHARE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="47" t="inlineStr">
+        <is>
+          <t>Things to NOT tell the guest:</t>
+        </is>
+      </c>
+      <c r="B21" s="48" t="n"/>
+      <c r="C21" s="48" t="n"/>
+      <c r="D21" s="101" t="inlineStr"/>
+      <c r="E21" s="48" t="n"/>
+      <c r="F21" s="48" t="n"/>
+      <c r="G21" s="48" t="n"/>
+      <c r="H21" s="48" t="n"/>
+      <c r="I21" s="48" t="n"/>
+      <c r="J21" s="48" t="n"/>
+      <c r="K21" s="48" t="n"/>
+      <c r="L21" s="50" t="n"/>
+    </row>
+    <row r="22" ht="12" customHeight="1">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
+      <c r="I22" s="6" t="n"/>
+      <c r="J22" s="6" t="n"/>
+      <c r="K22" s="6" t="n"/>
+      <c r="L22" s="6" t="n"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="102" t="inlineStr">
+        <is>
+          <t>Right-click this tab → Hide before saving or sharing. Excel: RIGHT-click tab → Hide. Google Sheets: right-click → Hide sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="27">
+    <mergeCell ref="D21:L21"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="D11:L11"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="D17:L17"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="D16:L16"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A1:L2"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D18:L18"/>
+    <mergeCell ref="D9:L9"/>
+    <mergeCell ref="A24:L25"/>
+    <mergeCell ref="D8:L8"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A20:L20"/>
+    <mergeCell ref="D15:L15"/>
+    <mergeCell ref="D14:L14"/>
+    <mergeCell ref="A13:L13"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D10:L10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A16:C16"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix: v2.1 Departure progress bug — exclude formula row from COUNTA
Departure's B9 is a formula (checkout day derived from Property!B11)
that COUNTA always counts as 'filled'. This inflated the Start-tab
progress dashboard for Departure: showed 1/6 on a blank form and
100% when 5 of 6 user inputs were filled.

While auditing the fix I also noticed the old B8:B13 range was missing
the custom_tasks cell at B16 entirely, so a completed checklist could
never show 100%. Both issues fixed by switching Departure's COUNTA to
an explicit multi-ref: COUNTA('Departure'!B8, 'Departure'!B10:B13,
'Departure'!B16) — skipping B9 (formula) and including B16 (custom
tasks). Applied to both the per-section status row on Start and the
overall-completion percentage formula.

Flagged by code reviewer on Task 1.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/_masters/GST-001-welcome-book-BLANK.xlsx
+++ b/templates/_masters/GST-001-welcome-book-BLANK.xlsx
@@ -1609,7 +1609,7 @@
         </is>
       </c>
       <c r="G36" s="16">
-        <f>TEXT((COUNTA('Property'!B8:B15) + COUNTA('Arrival'!B8:B14) + COUNTA('WiFi + Tech'!B8:B15) + COUNTA('House Rules'!B8:B14) + COUNTA('Local Guide'!B10:E29) + COUNTA('Trash'!B8:B14) + COUNTA('Departure'!B8:B13) + COUNTA('Emergency'!B8:B16))/132, "0%") &amp; " complete"</f>
+        <f>TEXT((COUNTA('Property'!B8:B15) + COUNTA('Arrival'!B8:B14) + COUNTA('WiFi + Tech'!B8:B15) + COUNTA('House Rules'!B8:B14) + COUNTA('Local Guide'!B10:E29) + COUNTA('Trash'!B8:B14) + COUNTA('Departure'!B8,'Departure'!B10:B13,'Departure'!B16) + COUNTA('Emergency'!B8:B16))/132, "0%") &amp; " complete"</f>
         <v/>
       </c>
     </row>
@@ -1710,7 +1710,7 @@
         </is>
       </c>
       <c r="G44" s="18">
-        <f>IF(COUNTA('Departure'!B8:B13)=6,"✅ Done",IF(COUNTA('Departure'!B8:B13)=0,"⏳ Empty","⏳ "&amp;COUNTA('Departure'!B8:B13)&amp;" of 6"))</f>
+        <f>IF(COUNTA('Departure'!B8,'Departure'!B10:B13,'Departure'!B16)=6,"✅ Done",IF(COUNTA('Departure'!B8,'Departure'!B10:B13,'Departure'!B16)=0,"⏳ Empty","⏳ "&amp;COUNTA('Departure'!B8,'Departure'!B10:B13,'Departure'!B16)&amp;" of 6"))</f>
         <v/>
       </c>
       <c r="K44" s="19">

</xml_diff>

<commit_message>
feat: v2.1 Launch tab replaces Review & Print
Tab 9 renamed Review & Print -> Launch. The 3-page live-preview
(rows 24-80 of v2) deleted -- preview moves to the HTML renderer.

Kept: readiness dashboard (rows 8-14, 3 cards with Completion %,
Red Flags, Status). The big pseudo-button is now labeled
OPEN YOUR WELCOME BOOK -> and uses a relative HYPERLINK to the
bundled welcome-book-renderer.html (same folder as xlsx).

brand_config.pseudo_button extended with external_link kwarg for
cross-file HYPERLINK formulas. Existing call sites unchanged.
</commit_message>
<xml_diff>
--- a/templates/_masters/GST-001-welcome-book-BLANK.xlsx
+++ b/templates/_masters/GST-001-welcome-book-BLANK.xlsx
@@ -16,7 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trash" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Departure" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emergency" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Print" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bonus" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="× Host Notes" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
@@ -24,7 +24,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Start'!$A$1:$L$52</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Local Guide'!$A$1:$E$33</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'Emergency'!$A$1:$L$21</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="9">'Review &amp; Print'!$A$24:$L$80</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="9">'Launch'!$A$1:$L$22</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="10">'Bonus'!$A$1:$L$20</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="11">'× Host Notes'!$A$1</definedName>
   </definedNames>
@@ -35,7 +35,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="50">
+  <fonts count="38">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -235,76 +235,6 @@
       <i val="1"/>
       <color rgb="006B7280"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="0012304E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="002B2B2B"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="0012304E"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="002B2B2B"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="0012304E"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="002B2B2B"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Georgia"/>
-      <b val="1"/>
-      <color rgb="0012304E"/>
-      <sz val="20"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="006B7280"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Georgia"/>
-      <b val="1"/>
-      <color rgb="0012304E"/>
-      <sz val="18"/>
-    </font>
-    <font>
-      <name val="Georgia"/>
-      <b val="1"/>
-      <color rgb="00B91C1C"/>
-      <sz val="18"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="0012304E"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="002B2B2B"/>
-      <sz val="14"/>
     </font>
     <font>
       <name val="Georgia"/>
@@ -618,7 +548,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -800,66 +730,20 @@
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="27" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="34" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="35" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="36" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -875,7 +759,7 @@
     <xf numFmtId="0" fontId="7" fillId="7" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="37" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1822,7 +1706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1855,14 +1739,14 @@
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="13">
-        <f>HYPERLINK("#'Emergency'!A5", "← BACK")</f>
+        <f>HYPERLINK("#'Emergency'!A5", "← BACK: Emergency")</f>
         <v/>
       </c>
       <c r="B2" s="14" t="n"/>
       <c r="C2" s="14" t="n"/>
       <c r="D2" s="61" t="inlineStr">
         <is>
-          <t>REVIEW &amp; PRINT</t>
+          <t>LAUNCH</t>
         </is>
       </c>
     </row>
@@ -1890,7 +1774,7 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>Preview below. Hit Print when happy.</t>
+          <t>Open it in the renderer, then save as PDF.</t>
         </is>
       </c>
     </row>
@@ -2041,8 +1925,7 @@
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="13">
-        <f>HYPERLINK("#'Review &amp; Print'!A24", "📄  GENERATE YOUR PDF
-Press Ctrl+P → choose 'Save as PDF'")</f>
+        <f>HYPERLINK("welcome-book-renderer.html", "📘  OPEN YOUR WELCOME BOOK →")</f>
         <v/>
       </c>
       <c r="B16" s="14" t="n"/>
@@ -2127,634 +2010,33 @@
       <c r="K21" s="14" t="n"/>
       <c r="L21" s="14" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="18" customHeight="1">
       <c r="A22" s="76" t="inlineStr">
         <is>
-          <t>Print area is pre-set to letter portrait. × Host Notes tab excluded.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="26">
-        <f>CONCATENATE("Welcome to ", Property!B8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1"/>
-    <row r="27">
-      <c r="A27" s="77" t="inlineStr">
-        <is>
-          <t>Host:</t>
-        </is>
-      </c>
-      <c r="E27" s="78">
-        <f>IF(Property!B9="","(not set)",Property!B9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="77" t="inlineStr">
-        <is>
-          <t>Host phone:</t>
-        </is>
-      </c>
-      <c r="E28" s="78">
-        <f>IF(Property!B10="","(not set)",Property!B10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="77" t="inlineStr">
-        <is>
-          <t>Check-in:</t>
-        </is>
-      </c>
-      <c r="E29" s="78">
-        <f>IF(Property!B11="","(not set)",Property!B11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="77" t="inlineStr">
-        <is>
-          <t>Check-out:</t>
-        </is>
-      </c>
-      <c r="E30" s="78">
-        <f>IF(Property!B12="","(not set)",Property!B12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="77" t="inlineStr">
-        <is>
-          <t>Address:</t>
-        </is>
-      </c>
-      <c r="E32" s="78">
-        <f>IF(Arrival!B8="","(not set)",Arrival!B8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="77" t="inlineStr">
-        <is>
-          <t>Entry method:</t>
-        </is>
-      </c>
-      <c r="E33" s="78">
-        <f>IF(Arrival!B9="","(not set)",Arrival!B9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="77" t="inlineStr">
-        <is>
-          <t>Door/lock code:</t>
-        </is>
-      </c>
-      <c r="E34" s="78">
-        <f>IF(Arrival!B10="","(not set)",Arrival!B10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="79" t="inlineStr">
-        <is>
-          <t>Parking:</t>
-        </is>
-      </c>
-      <c r="E35" s="80">
-        <f>IF(Arrival!B11="","(not set)",Arrival!B11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="81" t="inlineStr"/>
-      <c r="E37" s="82">
-        <f>IF(""="","(not set)","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="83" t="inlineStr">
-        <is>
-          <t>WiFi</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="84" t="inlineStr">
-        <is>
-          <t>Network:</t>
-        </is>
-      </c>
-      <c r="E39" s="85">
-        <f>IF('WiFi + Tech'!B8="","(not set)",'WiFi + Tech'!B8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="84" t="inlineStr">
-        <is>
-          <t>Password:</t>
-        </is>
-      </c>
-      <c r="E40" s="85">
-        <f>IF('WiFi + Tech'!B9="","(not set)",'WiFi + Tech'!B9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" ht="28" customHeight="1">
-      <c r="A48" s="86" t="inlineStr">
-        <is>
-          <t>House Rules</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="77" t="inlineStr">
-        <is>
-          <t>Quiet hours:</t>
-        </is>
-      </c>
-      <c r="E49" s="78">
-        <f>IF('House Rules'!B8="","(not set)",'House Rules'!B8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="77" t="inlineStr">
-        <is>
-          <t>Max guests:</t>
-        </is>
-      </c>
-      <c r="E50" s="78">
-        <f>IF('House Rules'!B9="","(not set)",'House Rules'!B9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="77" t="inlineStr">
-        <is>
-          <t>Smoking:</t>
-        </is>
-      </c>
-      <c r="E51" s="78">
-        <f>IF('House Rules'!B10="","(not set)",'House Rules'!B10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="77" t="inlineStr">
-        <is>
-          <t>Pets:</t>
-        </is>
-      </c>
-      <c r="E52" s="78">
-        <f>IF('House Rules'!B11="","(not set)",'House Rules'!B11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="77" t="inlineStr">
-        <is>
-          <t>Events:</t>
-        </is>
-      </c>
-      <c r="E53" s="78">
-        <f>IF('House Rules'!B12="","(not set)",'House Rules'!B12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="77" t="inlineStr">
-        <is>
-          <t>Shoes:</t>
-        </is>
-      </c>
-      <c r="E54" s="78">
-        <f>IF('House Rules'!B13="","(not set)",'House Rules'!B13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56" ht="28" customHeight="1">
-      <c r="A56" s="86" t="inlineStr">
-        <is>
-          <t>Local Guide — Our Top 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="87">
-        <f>'Local Guide'!A10</f>
-        <v/>
-      </c>
-      <c r="C57" s="88">
-        <f>IF('Local Guide'!B10="","",'Local Guide'!B10)</f>
-        <v/>
-      </c>
-      <c r="G57" s="89">
-        <f>IF('Local Guide'!C10="","",'Local Guide'!C10)</f>
-        <v/>
-      </c>
-      <c r="I57" s="90">
-        <f>IF('Local Guide'!E10="","",'Local Guide'!E10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="87">
-        <f>'Local Guide'!A11</f>
-        <v/>
-      </c>
-      <c r="C58" s="88">
-        <f>IF('Local Guide'!B11="","",'Local Guide'!B11)</f>
-        <v/>
-      </c>
-      <c r="G58" s="89">
-        <f>IF('Local Guide'!C11="","",'Local Guide'!C11)</f>
-        <v/>
-      </c>
-      <c r="I58" s="90">
-        <f>IF('Local Guide'!E11="","",'Local Guide'!E11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="87">
-        <f>'Local Guide'!A12</f>
-        <v/>
-      </c>
-      <c r="C59" s="88">
-        <f>IF('Local Guide'!B12="","",'Local Guide'!B12)</f>
-        <v/>
-      </c>
-      <c r="G59" s="89">
-        <f>IF('Local Guide'!C12="","",'Local Guide'!C12)</f>
-        <v/>
-      </c>
-      <c r="I59" s="90">
-        <f>IF('Local Guide'!E12="","",'Local Guide'!E12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="87">
-        <f>'Local Guide'!A13</f>
-        <v/>
-      </c>
-      <c r="C60" s="88">
-        <f>IF('Local Guide'!B13="","",'Local Guide'!B13)</f>
-        <v/>
-      </c>
-      <c r="G60" s="89">
-        <f>IF('Local Guide'!C13="","",'Local Guide'!C13)</f>
-        <v/>
-      </c>
-      <c r="I60" s="90">
-        <f>IF('Local Guide'!E13="","",'Local Guide'!E13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="87">
-        <f>'Local Guide'!A14</f>
-        <v/>
-      </c>
-      <c r="C61" s="88">
-        <f>IF('Local Guide'!B14="","",'Local Guide'!B14)</f>
-        <v/>
-      </c>
-      <c r="G61" s="89">
-        <f>IF('Local Guide'!C14="","",'Local Guide'!C14)</f>
-        <v/>
-      </c>
-      <c r="I61" s="90">
-        <f>IF('Local Guide'!E14="","",'Local Guide'!E14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="87">
-        <f>'Local Guide'!A15</f>
-        <v/>
-      </c>
-      <c r="C62" s="88">
-        <f>IF('Local Guide'!B15="","",'Local Guide'!B15)</f>
-        <v/>
-      </c>
-      <c r="G62" s="89">
-        <f>IF('Local Guide'!C15="","",'Local Guide'!C15)</f>
-        <v/>
-      </c>
-      <c r="I62" s="90">
-        <f>IF('Local Guide'!E15="","",'Local Guide'!E15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="87">
-        <f>'Local Guide'!A16</f>
-        <v/>
-      </c>
-      <c r="C63" s="88">
-        <f>IF('Local Guide'!B16="","",'Local Guide'!B16)</f>
-        <v/>
-      </c>
-      <c r="G63" s="89">
-        <f>IF('Local Guide'!C16="","",'Local Guide'!C16)</f>
-        <v/>
-      </c>
-      <c r="I63" s="90">
-        <f>IF('Local Guide'!E16="","",'Local Guide'!E16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="87">
-        <f>'Local Guide'!A17</f>
-        <v/>
-      </c>
-      <c r="C64" s="88">
-        <f>IF('Local Guide'!B17="","",'Local Guide'!B17)</f>
-        <v/>
-      </c>
-      <c r="G64" s="89">
-        <f>IF('Local Guide'!C17="","",'Local Guide'!C17)</f>
-        <v/>
-      </c>
-      <c r="I64" s="90">
-        <f>IF('Local Guide'!E17="","",'Local Guide'!E17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="87">
-        <f>'Local Guide'!A18</f>
-        <v/>
-      </c>
-      <c r="C65" s="88">
-        <f>IF('Local Guide'!B18="","",'Local Guide'!B18)</f>
-        <v/>
-      </c>
-      <c r="G65" s="89">
-        <f>IF('Local Guide'!C18="","",'Local Guide'!C18)</f>
-        <v/>
-      </c>
-      <c r="I65" s="90">
-        <f>IF('Local Guide'!E18="","",'Local Guide'!E18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="87">
-        <f>'Local Guide'!A19</f>
-        <v/>
-      </c>
-      <c r="C66" s="88">
-        <f>IF('Local Guide'!B19="","",'Local Guide'!B19)</f>
-        <v/>
-      </c>
-      <c r="G66" s="89">
-        <f>IF('Local Guide'!C19="","",'Local Guide'!C19)</f>
-        <v/>
-      </c>
-      <c r="I66" s="90">
-        <f>IF('Local Guide'!E19="","",'Local Guide'!E19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="91" t="inlineStr">
-        <is>
-          <t>Trash &amp; Maintenance</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="77" t="inlineStr">
-        <is>
-          <t>Pickup day:</t>
-        </is>
-      </c>
-      <c r="E69" s="78">
-        <f>IF('Trash'!B8="","(not set)",'Trash'!B8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="77" t="inlineStr">
-        <is>
-          <t>Bin location:</t>
-        </is>
-      </c>
-      <c r="E70" s="78">
-        <f>IF('Trash'!B9="","(not set)",'Trash'!B9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="91" t="inlineStr">
-        <is>
-          <t>Checkout</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="77" t="inlineStr">
-        <is>
-          <t>Time:</t>
-        </is>
-      </c>
-      <c r="E73" s="78">
-        <f>IF(Departure!B8="","(not set)",Departure!B8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="77" t="inlineStr">
-        <is>
-          <t>Linens:</t>
-        </is>
-      </c>
-      <c r="E74" s="78">
-        <f>IF(Departure!B10="","(not set)",Departure!B10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="77" t="inlineStr">
-        <is>
-          <t>Key return:</t>
-        </is>
-      </c>
-      <c r="E75" s="78">
-        <f>IF(Departure!B13="","(not set)",Departure!B13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="92" t="inlineStr">
-        <is>
-          <t>Emergency — Call 911 First</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="77" t="inlineStr">
-        <is>
-          <t>Hospital:</t>
-        </is>
-      </c>
-      <c r="E78" s="78">
-        <f>IF(Emergency!B8="","(not set)",Emergency!B8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="77" t="inlineStr">
-        <is>
-          <t>Hospital phone:</t>
-        </is>
-      </c>
-      <c r="E79" s="78">
-        <f>IF(Emergency!B9="","(not set)",Emergency!B9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="93" t="inlineStr">
-        <is>
-          <t>Host phone:</t>
-        </is>
-      </c>
-      <c r="E80" s="94">
-        <f>IF(Property!B10="","(not set)",Property!B10)</f>
-        <v/>
+          <t>Drag this xlsx onto the page that opens. Pick your theme, palette, and logo. Ctrl+P to save as PDF.</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="112">
-    <mergeCell ref="C61:F61"/>
-    <mergeCell ref="A64:B64"/>
-    <mergeCell ref="E33:L33"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="E35:L35"/>
-    <mergeCell ref="G57:H57"/>
-    <mergeCell ref="C62:F62"/>
-    <mergeCell ref="E28:L28"/>
-    <mergeCell ref="G66:H66"/>
-    <mergeCell ref="A73:D73"/>
-    <mergeCell ref="A51:D51"/>
-    <mergeCell ref="E69:L69"/>
-    <mergeCell ref="E78:L78"/>
-    <mergeCell ref="A70:D70"/>
-    <mergeCell ref="C64:F64"/>
-    <mergeCell ref="E30:L30"/>
-    <mergeCell ref="A54:D54"/>
-    <mergeCell ref="G58:H58"/>
-    <mergeCell ref="C63:F63"/>
-    <mergeCell ref="I10:L11"/>
-    <mergeCell ref="A77:L77"/>
-    <mergeCell ref="A10:D11"/>
-    <mergeCell ref="A62:B62"/>
-    <mergeCell ref="I66:L66"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="I58:L58"/>
-    <mergeCell ref="E54:L54"/>
-    <mergeCell ref="E32:L32"/>
-    <mergeCell ref="A33:D33"/>
+  <mergeCells count="15">
     <mergeCell ref="D2:L2"/>
-    <mergeCell ref="G59:H59"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="A53:D53"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="G61:H61"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="E79:L79"/>
-    <mergeCell ref="E73:L73"/>
+    <mergeCell ref="A16:L21"/>
     <mergeCell ref="A9:D9"/>
+    <mergeCell ref="E9:H9"/>
+    <mergeCell ref="I9:L9"/>
+    <mergeCell ref="A12:D12"/>
     <mergeCell ref="E12:H12"/>
     <mergeCell ref="A5:L5"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="G62:H62"/>
+    <mergeCell ref="I12:L12"/>
+    <mergeCell ref="E10:H11"/>
+    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="I10:L11"/>
+    <mergeCell ref="A10:D11"/>
+    <mergeCell ref="A2:C2"/>
     <mergeCell ref="A4:L4"/>
-    <mergeCell ref="E34:L34"/>
-    <mergeCell ref="A38:L38"/>
-    <mergeCell ref="I61:L61"/>
-    <mergeCell ref="E74:L74"/>
-    <mergeCell ref="A79:D79"/>
-    <mergeCell ref="I57:L57"/>
-    <mergeCell ref="E49:L49"/>
-    <mergeCell ref="G65:H65"/>
-    <mergeCell ref="A74:D74"/>
-    <mergeCell ref="A63:B63"/>
-    <mergeCell ref="G60:H60"/>
-    <mergeCell ref="E37:L37"/>
-    <mergeCell ref="A52:D52"/>
-    <mergeCell ref="C57:F57"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="I59:L59"/>
-    <mergeCell ref="C66:F66"/>
-    <mergeCell ref="I60:L60"/>
-    <mergeCell ref="I9:L9"/>
-    <mergeCell ref="A65:B65"/>
-    <mergeCell ref="A34:D34"/>
-    <mergeCell ref="E51:L51"/>
-    <mergeCell ref="A39:D39"/>
-    <mergeCell ref="A22:L22"/>
-    <mergeCell ref="A49:D49"/>
-    <mergeCell ref="C58:F58"/>
-    <mergeCell ref="A72:L72"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="A69:D69"/>
-    <mergeCell ref="A78:D78"/>
-    <mergeCell ref="C65:F65"/>
-    <mergeCell ref="E27:L27"/>
-    <mergeCell ref="G64:H64"/>
-    <mergeCell ref="A80:D80"/>
-    <mergeCell ref="A37:D37"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="G63:H63"/>
-    <mergeCell ref="I62:L62"/>
-    <mergeCell ref="C60:F60"/>
-    <mergeCell ref="E75:L75"/>
-    <mergeCell ref="E53:L53"/>
-    <mergeCell ref="A32:D32"/>
-    <mergeCell ref="E50:L50"/>
-    <mergeCell ref="A60:B60"/>
-    <mergeCell ref="I64:L64"/>
-    <mergeCell ref="E52:L52"/>
-    <mergeCell ref="A56:L56"/>
-    <mergeCell ref="I63:L63"/>
-    <mergeCell ref="E39:L39"/>
-    <mergeCell ref="E10:H11"/>
-    <mergeCell ref="A40:D40"/>
-    <mergeCell ref="E29:L29"/>
-    <mergeCell ref="I65:L65"/>
-    <mergeCell ref="A66:B66"/>
-    <mergeCell ref="A24:L25"/>
-    <mergeCell ref="E40:L40"/>
-    <mergeCell ref="A68:L68"/>
-    <mergeCell ref="E80:L80"/>
-    <mergeCell ref="E70:L70"/>
-    <mergeCell ref="A48:L48"/>
-    <mergeCell ref="A16:L21"/>
-    <mergeCell ref="A75:D75"/>
-    <mergeCell ref="E9:H9"/>
-    <mergeCell ref="A50:D50"/>
-    <mergeCell ref="I12:L12"/>
-    <mergeCell ref="C59:F59"/>
-    <mergeCell ref="A58:B58"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" paperSize="1" fitToHeight="3" fitToWidth="1"/>
-  <rowBreaks count="2" manualBreakCount="2">
-    <brk id="46" min="0" max="16383" man="1"/>
-    <brk id="66" min="0" max="16383" man="1"/>
-  </rowBreaks>
+  <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2783,55 +2065,55 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="95" t="n"/>
-      <c r="B1" s="95" t="n"/>
-      <c r="C1" s="95" t="n"/>
-      <c r="D1" s="95" t="n"/>
-      <c r="E1" s="95" t="n"/>
-      <c r="F1" s="95" t="n"/>
-      <c r="G1" s="95" t="n"/>
-      <c r="H1" s="95" t="n"/>
-      <c r="I1" s="95" t="n"/>
-      <c r="J1" s="95" t="n"/>
-      <c r="K1" s="95" t="n"/>
-      <c r="L1" s="95" t="n"/>
+      <c r="A1" s="77" t="n"/>
+      <c r="B1" s="77" t="n"/>
+      <c r="C1" s="77" t="n"/>
+      <c r="D1" s="77" t="n"/>
+      <c r="E1" s="77" t="n"/>
+      <c r="F1" s="77" t="n"/>
+      <c r="G1" s="77" t="n"/>
+      <c r="H1" s="77" t="n"/>
+      <c r="I1" s="77" t="n"/>
+      <c r="J1" s="77" t="n"/>
+      <c r="K1" s="77" t="n"/>
+      <c r="L1" s="77" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="45">
-        <f>HYPERLINK("#'Review &amp; Print'!A1", "← BACK")</f>
+        <f>HYPERLINK("#'Launch'!A1", "← BACK")</f>
         <v/>
       </c>
       <c r="B2" s="46" t="n"/>
       <c r="C2" s="46" t="n"/>
-      <c r="D2" s="96" t="inlineStr">
+      <c r="D2" s="78" t="inlineStr">
         <is>
           <t>BONUS</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="95" t="n"/>
-      <c r="B3" s="95" t="n"/>
-      <c r="C3" s="95" t="n"/>
-      <c r="D3" s="95" t="n"/>
-      <c r="E3" s="95" t="n"/>
-      <c r="F3" s="95" t="n"/>
-      <c r="G3" s="95" t="n"/>
-      <c r="H3" s="95" t="n"/>
-      <c r="I3" s="95" t="n"/>
-      <c r="J3" s="95" t="n"/>
-      <c r="K3" s="95" t="n"/>
-      <c r="L3" s="95" t="n"/>
+      <c r="A3" s="77" t="n"/>
+      <c r="B3" s="77" t="n"/>
+      <c r="C3" s="77" t="n"/>
+      <c r="D3" s="77" t="n"/>
+      <c r="E3" s="77" t="n"/>
+      <c r="F3" s="77" t="n"/>
+      <c r="G3" s="77" t="n"/>
+      <c r="H3" s="77" t="n"/>
+      <c r="I3" s="77" t="n"/>
+      <c r="J3" s="77" t="n"/>
+      <c r="K3" s="77" t="n"/>
+      <c r="L3" s="77" t="n"/>
     </row>
     <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="97" t="inlineStr">
+      <c r="A4" s="79" t="inlineStr">
         <is>
           <t>Bonus — Airbnb Listing Copy</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="98" t="inlineStr">
+      <c r="A5" s="80" t="inlineStr">
         <is>
           <t>Copy these blocks into your Airbnb listing — hosts using them see 40% better guest comprehension.</t>
         </is>
@@ -2866,7 +2148,7 @@
       </c>
     </row>
     <row r="10" ht="130" customHeight="1">
-      <c r="A10" s="99" t="inlineStr">
+      <c r="A10" s="81" t="inlineStr">
         <is>
           <t>We’re glad to have you. A few practical notes so everyone has a great stay:
 • Quiet hours from 10 PM to 7 AM — sound carries through the walls.
@@ -2897,7 +2179,7 @@
       </c>
     </row>
     <row r="13" ht="180" customHeight="1">
-      <c r="A13" s="99" t="inlineStr">
+      <c r="A13" s="81" t="inlineStr">
         <is>
           <t>Day-of check-in:
 1. The door uses a smart lock. Your code is 4321 (reset after checkout). 
@@ -2927,7 +2209,7 @@
       </c>
     </row>
     <row r="16" ht="160" customHeight="1">
-      <c r="A16" s="99" t="inlineStr">
+      <c r="A16" s="81" t="inlineStr">
         <is>
           <t>Hope your stay’s been great. Quick reminders for tomorrow:
 • Checkout is 11 AM sharp — we have a same-day turnover.
@@ -2953,7 +2235,7 @@
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="45">
-        <f>HYPERLINK("#'Review &amp; Print'!A1", "← Back: Review &amp; Print")</f>
+        <f>HYPERLINK("#'Launch'!A1", "← Back: Launch")</f>
         <v/>
       </c>
       <c r="B18" s="46" t="n"/>
@@ -3038,32 +2320,32 @@
     </row>
     <row r="2" ht="30" customHeight="1"/>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="100" t="inlineStr">
+      <c r="A3" s="82" t="inlineStr">
         <is>
           <t>Right-click this tab → 'Hide' before saving the workbook as a PDF or sharing with guests.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="101" t="inlineStr">
+      <c r="A4" s="83" t="inlineStr">
         <is>
           <t>This tab's Print Area is deliberately set to A1:A1 so if you accidentally print it, you get a near-empty page, not your private notes.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="102" t="n"/>
-      <c r="B5" s="102" t="n"/>
-      <c r="C5" s="102" t="n"/>
-      <c r="D5" s="102" t="n"/>
-      <c r="E5" s="102" t="n"/>
-      <c r="F5" s="102" t="n"/>
-      <c r="G5" s="102" t="n"/>
-      <c r="H5" s="102" t="n"/>
-      <c r="I5" s="102" t="n"/>
-      <c r="J5" s="102" t="n"/>
-      <c r="K5" s="102" t="n"/>
-      <c r="L5" s="102" t="n"/>
+      <c r="A5" s="84" t="n"/>
+      <c r="B5" s="84" t="n"/>
+      <c r="C5" s="84" t="n"/>
+      <c r="D5" s="84" t="n"/>
+      <c r="E5" s="84" t="n"/>
+      <c r="F5" s="84" t="n"/>
+      <c r="G5" s="84" t="n"/>
+      <c r="H5" s="84" t="n"/>
+      <c r="I5" s="84" t="n"/>
+      <c r="J5" s="84" t="n"/>
+      <c r="K5" s="84" t="n"/>
+      <c r="L5" s="84" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="29" t="inlineStr">
@@ -3080,7 +2362,7 @@
       </c>
       <c r="B8" s="32" t="n"/>
       <c r="C8" s="32" t="n"/>
-      <c r="D8" s="103" t="inlineStr"/>
+      <c r="D8" s="85" t="inlineStr"/>
       <c r="E8" s="32" t="n"/>
       <c r="F8" s="32" t="n"/>
       <c r="G8" s="32" t="n"/>
@@ -3134,7 +2416,7 @@
       </c>
       <c r="B11" s="42" t="n"/>
       <c r="C11" s="42" t="n"/>
-      <c r="D11" s="104" t="inlineStr"/>
+      <c r="D11" s="86" t="inlineStr"/>
       <c r="E11" s="42" t="n"/>
       <c r="F11" s="42" t="n"/>
       <c r="G11" s="42" t="n"/>
@@ -3173,7 +2455,7 @@
       </c>
       <c r="B14" s="32" t="n"/>
       <c r="C14" s="32" t="n"/>
-      <c r="D14" s="103" t="inlineStr"/>
+      <c r="D14" s="85" t="inlineStr"/>
       <c r="E14" s="32" t="n"/>
       <c r="F14" s="32" t="n"/>
       <c r="G14" s="32" t="n"/>
@@ -3245,7 +2527,7 @@
       </c>
       <c r="B18" s="42" t="n"/>
       <c r="C18" s="42" t="n"/>
-      <c r="D18" s="104" t="inlineStr"/>
+      <c r="D18" s="86" t="inlineStr"/>
       <c r="E18" s="42" t="n"/>
       <c r="F18" s="42" t="n"/>
       <c r="G18" s="42" t="n"/>
@@ -3284,7 +2566,7 @@
       </c>
       <c r="B21" s="52" t="n"/>
       <c r="C21" s="52" t="n"/>
-      <c r="D21" s="105" t="inlineStr"/>
+      <c r="D21" s="87" t="inlineStr"/>
       <c r="E21" s="52" t="n"/>
       <c r="F21" s="52" t="n"/>
       <c r="G21" s="52" t="n"/>
@@ -3309,7 +2591,7 @@
       <c r="L22" s="6" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="106" t="inlineStr">
+      <c r="A24" s="88" t="inlineStr">
         <is>
           <t>Right-click this tab → Hide before saving or sharing. Excel: RIGHT-click tab → Hide. Google Sheets: right-click → Hide sheet.</t>
         </is>
@@ -5784,7 +5066,7 @@
         </is>
       </c>
       <c r="J2" s="24">
-        <f>HYPERLINK("#'Review &amp; Print'!A1", "REVIEW →")</f>
+        <f>HYPERLINK("#'Launch'!A1", "LAUNCH →")</f>
         <v/>
       </c>
       <c r="K2" s="25" t="n"/>

</xml_diff>

<commit_message>
feat: GST-001 v2.2 — Safety & Disclosures tab
New input tab inserted between Departure and Emergency. Six fields
(B8:B13): recording devices (required, Airbnb policy compliance),
smoke + CO alarm locations, fire extinguisher, evacuation notes,
hazards, backup host contact. Empty fields suppress their renderer
row; an entirely empty block suppresses the heading too.

Renderer adds renderSafetyBlock invoked on page 3 above Emergency
across all three themes (Magazine card with accent rule, Editorial
typography, Hotel centered with DISCLOSURES subhead). 240-char
truncation + page-break-inside: avoid handle the §4.4 overflow case.

Spec: docs/superpowers/specs/2026-04-25-welcome-book-v2.2-safety-disclosures.md

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/_masters/GST-001-welcome-book-BLANK.xlsx
+++ b/templates/_masters/GST-001-welcome-book-BLANK.xlsx
@@ -15,18 +15,19 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local Guide" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trash" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Departure" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emergency" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bonus" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="× Host Notes" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Safety &amp; Disclosures" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emergency" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bonus" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="× Host Notes" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Start'!$A$1:$L$52</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Local Guide'!$A$1:$E$33</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="8">'Emergency'!$A$1:$L$21</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="9">'Launch'!$A$1:$L$22</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="10">'Bonus'!$A$1:$L$20</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="11">'× Host Notes'!$A$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="9">'Emergency'!$A$1:$L$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="10">'Launch'!$A$1:$L$22</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="11">'Bonus'!$A$1:$L$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="12">'× Host Notes'!$A$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1493,7 +1494,7 @@
         </is>
       </c>
       <c r="G36" s="16">
-        <f>TEXT((COUNTA('Property'!B8:B15) + COUNTA('Arrival'!B8:B14) + COUNTA('WiFi + Tech'!B8:B15) + COUNTA('House Rules'!B8:B14) + COUNTA('Local Guide'!B10:E29) + COUNTA('Trash'!B8:B14) + COUNTA('Departure'!B8,'Departure'!B10:B13,'Departure'!B16) + COUNTA('Emergency'!B8:B16))/132, "0%") &amp; " complete"</f>
+        <f>TEXT((COUNTA('Property'!B8:B15) + COUNTA('Arrival'!B8:B14) + COUNTA('WiFi + Tech'!B8:B15) + COUNTA('House Rules'!B8:B14) + COUNTA('Local Guide'!B10:E29) + COUNTA('Trash'!B8:B14) + COUNTA('Departure'!B8,'Departure'!B10:B13,'Departure'!B16) + COUNTA('Safety &amp; Disclosures'!B8:B13) + COUNTA('Emergency'!B8:B16))/138, "0%") &amp; " complete"</f>
         <v/>
       </c>
     </row>
@@ -1605,14 +1606,29 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="17" t="inlineStr">
         <is>
-          <t>⑧ Emergency</t>
+          <t>⑧ Safety &amp; Disclosures</t>
         </is>
       </c>
       <c r="G45" s="18">
+        <f>IF(COUNTA('Safety &amp; Disclosures'!B8:B13)=6,"✅ Done",IF(COUNTA('Safety &amp; Disclosures'!B8:B13)=0,"⏳ Empty","⏳ "&amp;COUNTA('Safety &amp; Disclosures'!B8:B13)&amp;" of 6"))</f>
+        <v/>
+      </c>
+      <c r="K45" s="19">
+        <f>HYPERLINK("#'Safety &amp; Disclosures'!A5","→ go")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="17" t="inlineStr">
+        <is>
+          <t>⑨ Emergency</t>
+        </is>
+      </c>
+      <c r="G46" s="18">
         <f>IF(COUNTA('Emergency'!B8:B16)=9,"✅ Done",IF(COUNTA('Emergency'!B8:B16)=0,"⏳ Empty","⏳ "&amp;COUNTA('Emergency'!B8:B16)&amp;" of 9"))</f>
         <v/>
       </c>
-      <c r="K45" s="19">
+      <c r="K46" s="19">
         <f>HYPERLINK("#'Emergency'!A5","→ go")</f>
         <v/>
       </c>
@@ -1646,9 +1662,10 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="46">
+  <mergeCells count="49">
     <mergeCell ref="A41:F41"/>
     <mergeCell ref="A7:L7"/>
+    <mergeCell ref="A46:F46"/>
     <mergeCell ref="B25:F25"/>
     <mergeCell ref="K45:L45"/>
     <mergeCell ref="A14:D18"/>
@@ -1660,6 +1677,7 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="I13:L13"/>
     <mergeCell ref="G40:J40"/>
+    <mergeCell ref="G46:J46"/>
     <mergeCell ref="A42:F42"/>
     <mergeCell ref="H25:L25"/>
     <mergeCell ref="A5:L5"/>
@@ -1667,6 +1685,7 @@
     <mergeCell ref="G43:J43"/>
     <mergeCell ref="K44:L44"/>
     <mergeCell ref="K41:L41"/>
+    <mergeCell ref="K46:L46"/>
     <mergeCell ref="K40:L40"/>
     <mergeCell ref="A4:L4"/>
     <mergeCell ref="G42:J42"/>
@@ -1700,6 +1719,353 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00F6EFE2"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="8" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="13">
+        <f>HYPERLINK("#'Safety &amp; Disclosures'!A5", "← BACK")</f>
+        <v/>
+      </c>
+      <c r="B2" s="14" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="23" t="inlineStr">
+        <is>
+          <t>SECTION 9 OF 9</t>
+        </is>
+      </c>
+      <c r="J2" s="24">
+        <f>HYPERLINK("#'Launch'!A1", "LAUNCH →")</f>
+        <v/>
+      </c>
+      <c r="K2" s="25" t="n"/>
+      <c r="L2" s="25" t="n"/>
+    </row>
+    <row r="3" ht="6" customHeight="1">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>Emergency Contacts</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>Keep this one nearby.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>911 first. Then the contacts below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="58" t="inlineStr">
+        <is>
+          <t>IN AN EMERGENCY — CALL 911</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>Nearest hospital:</t>
+        </is>
+      </c>
+      <c r="B8" s="31" t="n"/>
+      <c r="C8" s="32" t="n"/>
+      <c r="D8" s="32" t="n"/>
+      <c r="E8" s="32" t="n"/>
+      <c r="F8" s="32" t="n"/>
+      <c r="G8" s="32" t="n"/>
+      <c r="H8" s="32" t="n"/>
+      <c r="I8" s="32" t="n"/>
+      <c r="J8" s="32" t="n"/>
+      <c r="K8" s="32" t="n"/>
+      <c r="L8" s="33" t="n"/>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="34" t="inlineStr">
+        <is>
+          <t>Hospital phone:</t>
+        </is>
+      </c>
+      <c r="B9" s="35" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="6" t="n"/>
+      <c r="K9" s="6" t="n"/>
+      <c r="L9" s="36" t="n"/>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="34" t="inlineStr">
+        <is>
+          <t>Hospital address:</t>
+        </is>
+      </c>
+      <c r="B10" s="35" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="n"/>
+      <c r="K10" s="6" t="n"/>
+      <c r="L10" s="36" t="n"/>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="37" t="inlineStr">
+        <is>
+          <t>Urgent care:</t>
+        </is>
+      </c>
+      <c r="B11" s="38" t="n"/>
+      <c r="C11" s="39" t="n"/>
+      <c r="D11" s="39" t="n"/>
+      <c r="E11" s="39" t="n"/>
+      <c r="F11" s="39" t="n"/>
+      <c r="G11" s="39" t="n"/>
+      <c r="H11" s="39" t="n"/>
+      <c r="I11" s="39" t="n"/>
+      <c r="J11" s="39" t="n"/>
+      <c r="K11" s="39" t="n"/>
+      <c r="L11" s="40" t="n"/>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="34" t="inlineStr">
+        <is>
+          <t>Urgent care phone:</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="n"/>
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="36" t="n"/>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="34" t="inlineStr">
+        <is>
+          <t>Non-emergency police:</t>
+        </is>
+      </c>
+      <c r="B13" s="35" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="n"/>
+      <c r="K13" s="6" t="n"/>
+      <c r="L13" s="36" t="n"/>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="37" t="inlineStr">
+        <is>
+          <t>Poison control:</t>
+        </is>
+      </c>
+      <c r="B14" s="59" t="inlineStr">
+        <is>
+          <t>1-800-222-1222</t>
+        </is>
+      </c>
+      <c r="C14" s="39" t="n"/>
+      <c r="D14" s="39" t="n"/>
+      <c r="E14" s="39" t="n"/>
+      <c r="F14" s="39" t="n"/>
+      <c r="G14" s="39" t="n"/>
+      <c r="H14" s="39" t="n"/>
+      <c r="I14" s="39" t="n"/>
+      <c r="J14" s="39" t="n"/>
+      <c r="K14" s="39" t="n"/>
+      <c r="L14" s="40" t="n"/>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="34" t="inlineStr">
+        <is>
+          <t>24-hr vet (if pets):</t>
+        </is>
+      </c>
+      <c r="B15" s="35" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="36" t="n"/>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="34" t="inlineStr">
+        <is>
+          <t>Utility outage reporting:</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
+      <c r="J16" s="6" t="n"/>
+      <c r="K16" s="6" t="n"/>
+      <c r="L16" s="36" t="n"/>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="48" t="inlineStr">
+        <is>
+          <t>Host phone (call/text):</t>
+        </is>
+      </c>
+      <c r="B17" s="60">
+        <f>Property!B10</f>
+        <v/>
+      </c>
+      <c r="C17" s="42" t="n"/>
+      <c r="D17" s="42" t="n"/>
+      <c r="E17" s="42" t="n"/>
+      <c r="F17" s="42" t="n"/>
+      <c r="G17" s="42" t="n"/>
+      <c r="H17" s="42" t="n"/>
+      <c r="I17" s="42" t="n"/>
+      <c r="J17" s="42" t="n"/>
+      <c r="K17" s="42" t="n"/>
+      <c r="L17" s="43" t="n"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="45">
+        <f>HYPERLINK("#'Safety &amp; Disclosures'!A5", "← Back: Safety &amp; Disclosures")</f>
+        <v/>
+      </c>
+      <c r="B19" s="46" t="n"/>
+      <c r="C19" s="46" t="n"/>
+      <c r="D19" s="46" t="n"/>
+      <c r="E19" s="46" t="n"/>
+      <c r="F19" s="46" t="n"/>
+      <c r="G19" s="24">
+        <f>HYPERLINK("#'Launch'!A1", "Launch →")</f>
+        <v/>
+      </c>
+      <c r="H19" s="25" t="n"/>
+      <c r="I19" s="25" t="n"/>
+      <c r="J19" s="25" t="n"/>
+      <c r="K19" s="25" t="n"/>
+      <c r="L19" s="25" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="46" t="n"/>
+      <c r="B20" s="46" t="n"/>
+      <c r="C20" s="46" t="n"/>
+      <c r="D20" s="46" t="n"/>
+      <c r="E20" s="46" t="n"/>
+      <c r="F20" s="46" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="25" t="n"/>
+      <c r="I20" s="25" t="n"/>
+      <c r="J20" s="25" t="n"/>
+      <c r="K20" s="25" t="n"/>
+      <c r="L20" s="25" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="19">
+    <mergeCell ref="D2:I2"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="A19:F20"/>
+    <mergeCell ref="B16:L16"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="B12:L12"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="B11:L11"/>
+    <mergeCell ref="B14:L14"/>
+    <mergeCell ref="B17:L17"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="B8:L8"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="B13:L13"/>
+    <mergeCell ref="G19:L20"/>
+    <mergeCell ref="B10:L10"/>
+    <mergeCell ref="B9:L9"/>
+    <mergeCell ref="B15:L15"/>
+    <mergeCell ref="A6:L6"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C9A24B"/>
@@ -1834,21 +2200,21 @@
     </row>
     <row r="10">
       <c r="A10" s="67">
-        <f>TEXT((COUNTA('Property'!B8:B15) + COUNTA('Arrival'!B8:B14) + COUNTA('WiFi + Tech'!B8:B15) + COUNTA('House Rules'!B8:B14) + COUNTA('Local Guide'!B10:E29) + COUNTA('Trash'!B8:B14) + COUNTA('Departure'!B8:B13) + COUNTA('Emergency'!B8:B16))/132, "0%")</f>
+        <f>TEXT((COUNTA('Property'!B8:B15) + COUNTA('Arrival'!B8:B14) + COUNTA('WiFi + Tech'!B8:B15) + COUNTA('House Rules'!B8:B14) + COUNTA('Local Guide'!B10:E29) + COUNTA('Trash'!B8:B14) + COUNTA('Departure'!B8:B13) + COUNTA('Safety &amp; Disclosures'!B8:B13) + COUNTA('Emergency'!B8:B16))/138, "0%")</f>
         <v/>
       </c>
       <c r="B10" s="68" t="n"/>
       <c r="C10" s="68" t="n"/>
       <c r="D10" s="69" t="n"/>
       <c r="E10" s="70">
-        <f>IF('Property'!B8="",1,0) + IF('Property'!B9="",1,0) + IF('Property'!B10="",1,0) + IF('WiFi + Tech'!B8="",1,0) + IF('WiFi + Tech'!B9="",1,0) + IF('Trash'!B8="",1,0) + IF('Departure'!B8="",1,0) + IF('Emergency'!B8="",1,0) + IF('Emergency'!B9="",1,0) + IF('Emergency'!B11="",1,0)</f>
+        <f>IF('Property'!B8="",1,0) + IF('Property'!B9="",1,0) + IF('Property'!B10="",1,0) + IF('WiFi + Tech'!B8="",1,0) + IF('WiFi + Tech'!B9="",1,0) + IF('Trash'!B8="",1,0) + IF('Departure'!B8="",1,0) + IF('Safety &amp; Disclosures'!B8="",1,0) + IF('Emergency'!B8="",1,0) + IF('Emergency'!B9="",1,0) + IF('Emergency'!B11="",1,0)</f>
         <v/>
       </c>
       <c r="F10" s="68" t="n"/>
       <c r="G10" s="68" t="n"/>
       <c r="H10" s="69" t="n"/>
       <c r="I10" s="71">
-        <f>IF((IF('Property'!B8="",1,0) + IF('Property'!B9="",1,0) + IF('Property'!B10="",1,0) + IF('WiFi + Tech'!B8="",1,0) + IF('WiFi + Tech'!B9="",1,0) + IF('Trash'!B8="",1,0) + IF('Departure'!B8="",1,0) + IF('Emergency'!B8="",1,0) + IF('Emergency'!B9="",1,0) + IF('Emergency'!B11="",1,0))=0,"READY",IF((IF('Property'!B8="",1,0) + IF('Property'!B9="",1,0) + IF('Property'!B10="",1,0) + IF('WiFi + Tech'!B8="",1,0) + IF('WiFi + Tech'!B9="",1,0) + IF('Trash'!B8="",1,0) + IF('Departure'!B8="",1,0) + IF('Emergency'!B8="",1,0) + IF('Emergency'!B9="",1,0) + IF('Emergency'!B11="",1,0))&lt;=2,"MINOR","NEEDS WORK"))</f>
+        <f>IF((IF('Property'!B8="",1,0) + IF('Property'!B9="",1,0) + IF('Property'!B10="",1,0) + IF('WiFi + Tech'!B8="",1,0) + IF('WiFi + Tech'!B9="",1,0) + IF('Trash'!B8="",1,0) + IF('Departure'!B8="",1,0) + IF('Safety &amp; Disclosures'!B8="",1,0) + IF('Emergency'!B8="",1,0) + IF('Emergency'!B9="",1,0) + IF('Emergency'!B11="",1,0))=0,"READY",IF((IF('Property'!B8="",1,0) + IF('Property'!B9="",1,0) + IF('Property'!B10="",1,0) + IF('WiFi + Tech'!B8="",1,0) + IF('WiFi + Tech'!B9="",1,0) + IF('Trash'!B8="",1,0) + IF('Departure'!B8="",1,0) + IF('Safety &amp; Disclosures'!B8="",1,0) + IF('Emergency'!B8="",1,0) + IF('Emergency'!B9="",1,0) + IF('Emergency'!B11="",1,0))&lt;=2,"MINOR","NEEDS WORK"))</f>
         <v/>
       </c>
       <c r="J10" s="68" t="n"/>
@@ -1872,7 +2238,7 @@
     <row r="12">
       <c r="A12" s="73" t="inlineStr">
         <is>
-          <t>of 132 fields filled</t>
+          <t>of 138 fields filled</t>
         </is>
       </c>
       <c r="B12" s="74" t="n"/>
@@ -2040,7 +2406,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00E2C884"/>
@@ -2287,7 +2653,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00B5725E"/>
@@ -2680,7 +3046,7 @@
       <c r="C2" s="14" t="n"/>
       <c r="D2" s="23" t="inlineStr">
         <is>
-          <t>SECTION 1 OF 8</t>
+          <t>SECTION 1 OF 9</t>
         </is>
       </c>
       <c r="J2" s="24">
@@ -3019,7 +3385,7 @@
       <c r="C2" s="14" t="n"/>
       <c r="D2" s="23" t="inlineStr">
         <is>
-          <t>SECTION 2 OF 8</t>
+          <t>SECTION 2 OF 9</t>
         </is>
       </c>
       <c r="J2" s="24">
@@ -3396,7 +3762,7 @@
       <c r="C2" s="14" t="n"/>
       <c r="D2" s="23" t="inlineStr">
         <is>
-          <t>SECTION 3 OF 8</t>
+          <t>SECTION 3 OF 9</t>
         </is>
       </c>
       <c r="J2" s="24">
@@ -3711,7 +4077,7 @@
       <c r="C2" s="14" t="n"/>
       <c r="D2" s="23" t="inlineStr">
         <is>
-          <t>SECTION 4 OF 8</t>
+          <t>SECTION 4 OF 9</t>
         </is>
       </c>
       <c r="J2" s="24">
@@ -4021,7 +4387,7 @@
       <c r="C2" s="14" t="n"/>
       <c r="D2" s="23" t="inlineStr">
         <is>
-          <t>SECTION 5 OF 8</t>
+          <t>SECTION 5 OF 9</t>
         </is>
       </c>
       <c r="J2" s="24">
@@ -4424,7 +4790,7 @@
       <c r="C2" s="14" t="n"/>
       <c r="D2" s="23" t="inlineStr">
         <is>
-          <t>SECTION 6 OF 8</t>
+          <t>SECTION 6 OF 9</t>
         </is>
       </c>
       <c r="J2" s="24">
@@ -4725,11 +5091,11 @@
       <c r="C2" s="14" t="n"/>
       <c r="D2" s="23" t="inlineStr">
         <is>
-          <t>SECTION 7 OF 8</t>
+          <t>SECTION 7 OF 9</t>
         </is>
       </c>
       <c r="J2" s="24">
-        <f>HYPERLINK("#'Emergency'!A5", "NEXT →")</f>
+        <f>HYPERLINK("#'Safety &amp; Disclosures'!A5", "NEXT →")</f>
         <v/>
       </c>
       <c r="K2" s="25" t="n"/>
@@ -4967,7 +5333,7 @@
       <c r="E18" s="46" t="n"/>
       <c r="F18" s="46" t="n"/>
       <c r="G18" s="45">
-        <f>HYPERLINK("#'Emergency'!A5", "Next: Emergency →")</f>
+        <f>HYPERLINK("#'Safety &amp; Disclosures'!A5", "Next: Safety &amp; Disclosures →")</f>
         <v/>
       </c>
       <c r="H18" s="46" t="n"/>
@@ -5022,7 +5388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5062,11 +5428,11 @@
       <c r="C2" s="14" t="n"/>
       <c r="D2" s="23" t="inlineStr">
         <is>
-          <t>SECTION 8 OF 8</t>
+          <t>SECTION 8 OF 9</t>
         </is>
       </c>
       <c r="J2" s="24">
-        <f>HYPERLINK("#'Launch'!A1", "LAUNCH →")</f>
+        <f>HYPERLINK("#'Emergency'!A5", "NEXT →")</f>
         <v/>
       </c>
       <c r="K2" s="25" t="n"/>
@@ -5089,35 +5455,35 @@
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>Emergency Contacts</t>
+          <t>Safety &amp; Disclosures</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>Keep this one nearby.</t>
+          <t>Disclosure first, then safety locations.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="28" t="inlineStr">
         <is>
-          <t>911 first. Then the contacts below.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="58" t="inlineStr">
-        <is>
-          <t>IN AN EMERGENCY — CALL 911</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="24" customHeight="1">
+          <t>Fill the highlighted fields below. The 'Launch' tab (last) shows what your guest will see.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>SAFETY &amp; DISCLOSURES</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
       <c r="A8" s="30" t="inlineStr">
         <is>
-          <t>Nearest hospital:</t>
+          <t>• Recording devices on property:</t>
         </is>
       </c>
       <c r="B8" s="31" t="n"/>
@@ -5132,28 +5498,28 @@
       <c r="K8" s="32" t="n"/>
       <c r="L8" s="33" t="n"/>
     </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="34" t="inlineStr">
-        <is>
-          <t>Hospital phone:</t>
-        </is>
-      </c>
-      <c r="B9" s="35" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="6" t="n"/>
-      <c r="J9" s="6" t="n"/>
-      <c r="K9" s="6" t="n"/>
-      <c r="L9" s="36" t="n"/>
-    </row>
-    <row r="10" ht="24" customHeight="1">
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="37" t="inlineStr">
+        <is>
+          <t>Smoke + CO alarm locations:</t>
+        </is>
+      </c>
+      <c r="B9" s="38" t="n"/>
+      <c r="C9" s="39" t="n"/>
+      <c r="D9" s="39" t="n"/>
+      <c r="E9" s="39" t="n"/>
+      <c r="F9" s="39" t="n"/>
+      <c r="G9" s="39" t="n"/>
+      <c r="H9" s="39" t="n"/>
+      <c r="I9" s="39" t="n"/>
+      <c r="J9" s="39" t="n"/>
+      <c r="K9" s="39" t="n"/>
+      <c r="L9" s="40" t="n"/>
+    </row>
+    <row r="10" ht="36" customHeight="1">
       <c r="A10" s="34" t="inlineStr">
         <is>
-          <t>Hospital address:</t>
+          <t>Fire extinguisher location:</t>
         </is>
       </c>
       <c r="B10" s="35" t="n"/>
@@ -5168,10 +5534,10 @@
       <c r="K10" s="6" t="n"/>
       <c r="L10" s="36" t="n"/>
     </row>
-    <row r="11" ht="24" customHeight="1">
+    <row r="11" ht="48" customHeight="1">
       <c r="A11" s="37" t="inlineStr">
         <is>
-          <t>Urgent care:</t>
+          <t>If you need to evacuate:</t>
         </is>
       </c>
       <c r="B11" s="38" t="n"/>
@@ -5186,10 +5552,10 @@
       <c r="K11" s="39" t="n"/>
       <c r="L11" s="40" t="n"/>
     </row>
-    <row r="12" ht="24" customHeight="1">
+    <row r="12" ht="48" customHeight="1">
       <c r="A12" s="34" t="inlineStr">
         <is>
-          <t>Urgent care phone:</t>
+          <t>Known hazards / things to know:</t>
         </is>
       </c>
       <c r="B12" s="35" t="n"/>
@@ -5205,159 +5571,89 @@
       <c r="L12" s="36" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="34" t="inlineStr">
-        <is>
-          <t>Non-emergency police:</t>
-        </is>
-      </c>
-      <c r="B13" s="35" t="n"/>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="6" t="n"/>
-      <c r="H13" s="6" t="n"/>
-      <c r="I13" s="6" t="n"/>
-      <c r="J13" s="6" t="n"/>
-      <c r="K13" s="6" t="n"/>
-      <c r="L13" s="36" t="n"/>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="37" t="inlineStr">
-        <is>
-          <t>Poison control:</t>
-        </is>
-      </c>
-      <c r="B14" s="59" t="inlineStr">
-        <is>
-          <t>1-800-222-1222</t>
-        </is>
-      </c>
-      <c r="C14" s="39" t="n"/>
-      <c r="D14" s="39" t="n"/>
-      <c r="E14" s="39" t="n"/>
-      <c r="F14" s="39" t="n"/>
-      <c r="G14" s="39" t="n"/>
-      <c r="H14" s="39" t="n"/>
-      <c r="I14" s="39" t="n"/>
-      <c r="J14" s="39" t="n"/>
-      <c r="K14" s="39" t="n"/>
-      <c r="L14" s="40" t="n"/>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="34" t="inlineStr">
-        <is>
-          <t>24-hr vet (if pets):</t>
-        </is>
-      </c>
-      <c r="B15" s="35" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="6" t="n"/>
-      <c r="I15" s="6" t="n"/>
-      <c r="J15" s="6" t="n"/>
-      <c r="K15" s="6" t="n"/>
-      <c r="L15" s="36" t="n"/>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="34" t="inlineStr">
-        <is>
-          <t>Utility outage reporting:</t>
-        </is>
-      </c>
-      <c r="B16" s="35" t="n"/>
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="6" t="n"/>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="6" t="n"/>
-      <c r="H16" s="6" t="n"/>
-      <c r="I16" s="6" t="n"/>
-      <c r="J16" s="6" t="n"/>
-      <c r="K16" s="6" t="n"/>
-      <c r="L16" s="36" t="n"/>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="48" t="inlineStr">
-        <is>
-          <t>Host phone (call/text):</t>
-        </is>
-      </c>
-      <c r="B17" s="60">
-        <f>Property!B10</f>
-        <v/>
-      </c>
-      <c r="C17" s="42" t="n"/>
-      <c r="D17" s="42" t="n"/>
-      <c r="E17" s="42" t="n"/>
-      <c r="F17" s="42" t="n"/>
-      <c r="G17" s="42" t="n"/>
-      <c r="H17" s="42" t="n"/>
-      <c r="I17" s="42" t="n"/>
-      <c r="J17" s="42" t="n"/>
-      <c r="K17" s="42" t="n"/>
-      <c r="L17" s="43" t="n"/>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="45">
+      <c r="A13" s="50" t="inlineStr">
+        <is>
+          <t>Backup host (if primary unreachable):</t>
+        </is>
+      </c>
+      <c r="B13" s="51" t="n"/>
+      <c r="C13" s="52" t="n"/>
+      <c r="D13" s="52" t="n"/>
+      <c r="E13" s="52" t="n"/>
+      <c r="F13" s="52" t="n"/>
+      <c r="G13" s="52" t="n"/>
+      <c r="H13" s="52" t="n"/>
+      <c r="I13" s="52" t="n"/>
+      <c r="J13" s="52" t="n"/>
+      <c r="K13" s="52" t="n"/>
+      <c r="L13" s="53" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="44" t="n"/>
+      <c r="B14" s="44" t="n"/>
+      <c r="C14" s="44" t="n"/>
+      <c r="D14" s="44" t="n"/>
+      <c r="E14" s="44" t="n"/>
+      <c r="F14" s="44" t="n"/>
+      <c r="G14" s="44" t="n"/>
+      <c r="H14" s="44" t="n"/>
+      <c r="I14" s="44" t="n"/>
+      <c r="J14" s="44" t="n"/>
+      <c r="K14" s="44" t="n"/>
+      <c r="L14" s="44" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="45">
         <f>HYPERLINK("#'Departure'!A5", "← Back: Departure")</f>
         <v/>
       </c>
-      <c r="B19" s="46" t="n"/>
-      <c r="C19" s="46" t="n"/>
-      <c r="D19" s="46" t="n"/>
-      <c r="E19" s="46" t="n"/>
-      <c r="F19" s="46" t="n"/>
-      <c r="G19" s="24">
-        <f>HYPERLINK("#'Launch'!A1", "Launch →")</f>
-        <v/>
-      </c>
-      <c r="H19" s="25" t="n"/>
-      <c r="I19" s="25" t="n"/>
-      <c r="J19" s="25" t="n"/>
-      <c r="K19" s="25" t="n"/>
-      <c r="L19" s="25" t="n"/>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="46" t="n"/>
-      <c r="B20" s="46" t="n"/>
-      <c r="C20" s="46" t="n"/>
-      <c r="D20" s="46" t="n"/>
-      <c r="E20" s="46" t="n"/>
-      <c r="F20" s="46" t="n"/>
-      <c r="G20" s="25" t="n"/>
-      <c r="H20" s="25" t="n"/>
-      <c r="I20" s="25" t="n"/>
-      <c r="J20" s="25" t="n"/>
-      <c r="K20" s="25" t="n"/>
-      <c r="L20" s="25" t="n"/>
+      <c r="B15" s="46" t="n"/>
+      <c r="C15" s="46" t="n"/>
+      <c r="D15" s="46" t="n"/>
+      <c r="E15" s="46" t="n"/>
+      <c r="F15" s="46" t="n"/>
+      <c r="G15" s="45">
+        <f>HYPERLINK("#'Emergency'!A5", "Next: Emergency →")</f>
+        <v/>
+      </c>
+      <c r="H15" s="46" t="n"/>
+      <c r="I15" s="46" t="n"/>
+      <c r="J15" s="46" t="n"/>
+      <c r="K15" s="46" t="n"/>
+      <c r="L15" s="46" t="n"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="46" t="n"/>
+      <c r="B16" s="46" t="n"/>
+      <c r="C16" s="46" t="n"/>
+      <c r="D16" s="46" t="n"/>
+      <c r="E16" s="46" t="n"/>
+      <c r="F16" s="46" t="n"/>
+      <c r="G16" s="46" t="n"/>
+      <c r="H16" s="46" t="n"/>
+      <c r="I16" s="46" t="n"/>
+      <c r="J16" s="46" t="n"/>
+      <c r="K16" s="46" t="n"/>
+      <c r="L16" s="46" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="15">
+    <mergeCell ref="J2:L2"/>
     <mergeCell ref="D2:I2"/>
     <mergeCell ref="A7:L7"/>
-    <mergeCell ref="A19:F20"/>
-    <mergeCell ref="B16:L16"/>
-    <mergeCell ref="A2:C2"/>
     <mergeCell ref="B12:L12"/>
+    <mergeCell ref="B13:L13"/>
+    <mergeCell ref="G15:L16"/>
+    <mergeCell ref="B9:L9"/>
     <mergeCell ref="A5:L5"/>
     <mergeCell ref="B11:L11"/>
-    <mergeCell ref="B14:L14"/>
-    <mergeCell ref="B17:L17"/>
+    <mergeCell ref="A6:L6"/>
+    <mergeCell ref="B10:L10"/>
+    <mergeCell ref="A15:F16"/>
+    <mergeCell ref="A2:C2"/>
     <mergeCell ref="A4:L4"/>
     <mergeCell ref="B8:L8"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="B13:L13"/>
-    <mergeCell ref="G19:L20"/>
-    <mergeCell ref="B10:L10"/>
-    <mergeCell ref="B9:L9"/>
-    <mergeCell ref="B15:L15"/>
-    <mergeCell ref="A6:L6"/>
   </mergeCells>
-  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" paperSize="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>